<commit_message>
re-source a granel - 355
</commit_message>
<xml_diff>
--- a/PLANILHA-FOTOS-NOVAS-355.xlsx
+++ b/PLANILHA-FOTOS-NOVAS-355.xlsx
@@ -678,7 +678,7 @@
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/adocantes-naturais/11511.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/adocantes-naturais/11511.webp</t>
         </is>
       </c>
     </row>
@@ -755,7 +755,7 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/adocantes-naturais/11817.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/adocantes-naturais/11817.png</t>
         </is>
       </c>
     </row>
@@ -832,7 +832,7 @@
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/adocantes-naturais/12026.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/adocantes-naturais/12026.jpg</t>
         </is>
       </c>
     </row>
@@ -909,7 +909,7 @@
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/adocantes-naturais/12027.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/adocantes-naturais/12027.webp</t>
         </is>
       </c>
     </row>
@@ -986,7 +986,7 @@
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/adocantes-naturais/12028.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/adocantes-naturais/12028.webp</t>
         </is>
       </c>
     </row>
@@ -1063,7 +1063,7 @@
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/adocantes-naturais/12174.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/adocantes-naturais/12174.webp</t>
         </is>
       </c>
     </row>
@@ -1140,7 +1140,7 @@
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10043.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10043.webp</t>
         </is>
       </c>
     </row>
@@ -1217,7 +1217,7 @@
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10092.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10092.webp</t>
         </is>
       </c>
     </row>
@@ -1294,7 +1294,7 @@
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10115.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10115.webp</t>
         </is>
       </c>
     </row>
@@ -1371,7 +1371,7 @@
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10217.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10217.webp</t>
         </is>
       </c>
     </row>
@@ -1448,7 +1448,7 @@
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10255.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10255.jpg</t>
         </is>
       </c>
     </row>
@@ -1525,7 +1525,7 @@
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10364.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10364.webp</t>
         </is>
       </c>
     </row>
@@ -1602,7 +1602,7 @@
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10395.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10395.webp</t>
         </is>
       </c>
     </row>
@@ -1679,7 +1679,7 @@
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10396.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10396.webp</t>
         </is>
       </c>
     </row>
@@ -1756,7 +1756,7 @@
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10652.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10652.webp</t>
         </is>
       </c>
     </row>
@@ -1833,7 +1833,7 @@
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10745.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10745.webp</t>
         </is>
       </c>
     </row>
@@ -1910,7 +1910,7 @@
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10866.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10866.webp</t>
         </is>
       </c>
     </row>
@@ -1987,7 +1987,7 @@
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10877.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10877.webp</t>
         </is>
       </c>
     </row>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10900.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10900.webp</t>
         </is>
       </c>
     </row>
@@ -2218,7 +2218,7 @@
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10910.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10910.webp</t>
         </is>
       </c>
     </row>
@@ -2295,7 +2295,7 @@
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10914.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10914.webp</t>
         </is>
       </c>
     </row>
@@ -2372,7 +2372,7 @@
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10915.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10915.webp</t>
         </is>
       </c>
     </row>
@@ -2449,7 +2449,7 @@
       </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10946.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10946.webp</t>
         </is>
       </c>
     </row>
@@ -2526,7 +2526,7 @@
       </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10957.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10957.webp</t>
         </is>
       </c>
     </row>
@@ -2603,7 +2603,7 @@
       </c>
       <c r="V28" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10978.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10978.webp</t>
         </is>
       </c>
     </row>
@@ -2680,7 +2680,7 @@
       </c>
       <c r="V29" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11005.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11005.webp</t>
         </is>
       </c>
     </row>
@@ -2757,7 +2757,7 @@
       </c>
       <c r="V30" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11054.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11054.jpg</t>
         </is>
       </c>
     </row>
@@ -2834,7 +2834,7 @@
       </c>
       <c r="V31" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11055.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11055.webp</t>
         </is>
       </c>
     </row>
@@ -2911,7 +2911,7 @@
       </c>
       <c r="V32" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11059.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11059.webp</t>
         </is>
       </c>
     </row>
@@ -2988,7 +2988,7 @@
       </c>
       <c r="V33" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11061.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11061.webp</t>
         </is>
       </c>
     </row>
@@ -3065,7 +3065,7 @@
       </c>
       <c r="V34" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11062.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11062.webp</t>
         </is>
       </c>
     </row>
@@ -3142,7 +3142,7 @@
       </c>
       <c r="V35" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11077.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11077.webp</t>
         </is>
       </c>
     </row>
@@ -3219,7 +3219,7 @@
       </c>
       <c r="V36" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11091.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11091.webp</t>
         </is>
       </c>
     </row>
@@ -3373,7 +3373,7 @@
       </c>
       <c r="V38" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11110.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11110.webp</t>
         </is>
       </c>
     </row>
@@ -3450,7 +3450,7 @@
       </c>
       <c r="V39" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11116.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11116.webp</t>
         </is>
       </c>
     </row>
@@ -3604,7 +3604,7 @@
       </c>
       <c r="V41" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11121.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11121.webp</t>
         </is>
       </c>
     </row>
@@ -3681,7 +3681,7 @@
       </c>
       <c r="V42" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11124.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11124.png</t>
         </is>
       </c>
     </row>
@@ -3758,7 +3758,7 @@
       </c>
       <c r="V43" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11125.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11125.webp</t>
         </is>
       </c>
     </row>
@@ -3835,7 +3835,7 @@
       </c>
       <c r="V44" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11132.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11132.webp</t>
         </is>
       </c>
     </row>
@@ -3912,7 +3912,7 @@
       </c>
       <c r="V45" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11136.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11136.webp</t>
         </is>
       </c>
     </row>
@@ -3989,7 +3989,7 @@
       </c>
       <c r="V46" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11137.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11137.webp</t>
         </is>
       </c>
     </row>
@@ -4066,7 +4066,7 @@
       </c>
       <c r="V47" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11160.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11160.webp</t>
         </is>
       </c>
     </row>
@@ -4143,7 +4143,7 @@
       </c>
       <c r="V48" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11175.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11175.webp</t>
         </is>
       </c>
     </row>
@@ -4220,7 +4220,7 @@
       </c>
       <c r="V49" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11259.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11259.webp</t>
         </is>
       </c>
     </row>
@@ -4374,7 +4374,7 @@
       </c>
       <c r="V51" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11325.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11325.webp</t>
         </is>
       </c>
     </row>
@@ -4451,7 +4451,7 @@
       </c>
       <c r="V52" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11326.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11326.webp</t>
         </is>
       </c>
     </row>
@@ -4528,7 +4528,7 @@
       </c>
       <c r="V53" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11329.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11329.jpg</t>
         </is>
       </c>
     </row>
@@ -4605,7 +4605,7 @@
       </c>
       <c r="V54" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11331.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11331.webp</t>
         </is>
       </c>
     </row>
@@ -4682,7 +4682,7 @@
       </c>
       <c r="V55" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11332.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11332.webp</t>
         </is>
       </c>
     </row>
@@ -4759,7 +4759,7 @@
       </c>
       <c r="V56" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11334.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11334.webp</t>
         </is>
       </c>
     </row>
@@ -4836,7 +4836,7 @@
       </c>
       <c r="V57" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11335.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11335.jpg</t>
         </is>
       </c>
     </row>
@@ -4913,7 +4913,7 @@
       </c>
       <c r="V58" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11337.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11337.webp</t>
         </is>
       </c>
     </row>
@@ -4990,7 +4990,7 @@
       </c>
       <c r="V59" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11338.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11338.webp</t>
         </is>
       </c>
     </row>
@@ -5144,7 +5144,7 @@
       </c>
       <c r="V61" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11340.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11340.webp</t>
         </is>
       </c>
     </row>
@@ -5221,7 +5221,7 @@
       </c>
       <c r="V62" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11341.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11341.webp</t>
         </is>
       </c>
     </row>
@@ -5298,7 +5298,7 @@
       </c>
       <c r="V63" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11342.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11342.webp</t>
         </is>
       </c>
     </row>
@@ -5375,7 +5375,7 @@
       </c>
       <c r="V64" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11400.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11400.jpg</t>
         </is>
       </c>
     </row>
@@ -5452,7 +5452,7 @@
       </c>
       <c r="V65" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11401.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11401.webp</t>
         </is>
       </c>
     </row>
@@ -5683,7 +5683,7 @@
       </c>
       <c r="V68" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/12052.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/12052.webp</t>
         </is>
       </c>
     </row>
@@ -5760,7 +5760,7 @@
       </c>
       <c r="V69" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/12091.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/12091.webp</t>
         </is>
       </c>
     </row>
@@ -6145,7 +6145,7 @@
       </c>
       <c r="V74" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/10037.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/10037.webp</t>
         </is>
       </c>
     </row>
@@ -6222,7 +6222,7 @@
       </c>
       <c r="V75" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/10044.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/10044.webp</t>
         </is>
       </c>
     </row>
@@ -6299,7 +6299,7 @@
       </c>
       <c r="V76" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/10068.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/10068.webp</t>
         </is>
       </c>
     </row>
@@ -6376,7 +6376,7 @@
       </c>
       <c r="V77" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/10073.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/10073.webp</t>
         </is>
       </c>
     </row>
@@ -6607,7 +6607,7 @@
       </c>
       <c r="V80" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11803.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11803.png</t>
         </is>
       </c>
     </row>
@@ -6684,7 +6684,7 @@
       </c>
       <c r="V81" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11848.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11848.webp</t>
         </is>
       </c>
     </row>
@@ -6761,7 +6761,7 @@
       </c>
       <c r="V82" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11861.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11861.webp</t>
         </is>
       </c>
     </row>
@@ -6838,7 +6838,7 @@
       </c>
       <c r="V83" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11902.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11902.webp</t>
         </is>
       </c>
     </row>
@@ -6915,7 +6915,7 @@
       </c>
       <c r="V84" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11939.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11939.webp</t>
         </is>
       </c>
     </row>
@@ -6992,7 +6992,7 @@
       </c>
       <c r="V85" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11996.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11996.webp</t>
         </is>
       </c>
     </row>
@@ -7069,7 +7069,7 @@
       </c>
       <c r="V86" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11998.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11998.webp</t>
         </is>
       </c>
     </row>
@@ -7146,7 +7146,7 @@
       </c>
       <c r="V87" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/12039.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/12039.webp</t>
         </is>
       </c>
     </row>
@@ -7223,7 +7223,7 @@
       </c>
       <c r="V88" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/12071.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/12071.webp</t>
         </is>
       </c>
     </row>
@@ -7300,7 +7300,7 @@
       </c>
       <c r="V89" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/12086.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/12086.webp</t>
         </is>
       </c>
     </row>
@@ -7377,7 +7377,7 @@
       </c>
       <c r="V90" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/12072.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/12072.png</t>
         </is>
       </c>
     </row>
@@ -7454,7 +7454,7 @@
       </c>
       <c r="V91" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/10277.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/10277.webp</t>
         </is>
       </c>
     </row>
@@ -7531,7 +7531,7 @@
       </c>
       <c r="V92" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/10278.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/10278.webp</t>
         </is>
       </c>
     </row>
@@ -7608,7 +7608,7 @@
       </c>
       <c r="V93" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/10873.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/10873.webp</t>
         </is>
       </c>
     </row>
@@ -7685,7 +7685,7 @@
       </c>
       <c r="V94" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/11480.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/11480.webp</t>
         </is>
       </c>
     </row>
@@ -7762,7 +7762,7 @@
       </c>
       <c r="V95" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/11895.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/11895.webp</t>
         </is>
       </c>
     </row>
@@ -7839,7 +7839,7 @@
       </c>
       <c r="V96" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/11898.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/11898.webp</t>
         </is>
       </c>
     </row>
@@ -7916,7 +7916,7 @@
       </c>
       <c r="V97" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/11940.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/11940.webp</t>
         </is>
       </c>
     </row>
@@ -7993,7 +7993,7 @@
       </c>
       <c r="V98" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/11941.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/11941.webp</t>
         </is>
       </c>
     </row>
@@ -8224,7 +8224,7 @@
       </c>
       <c r="V101" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/10944.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/10944.webp</t>
         </is>
       </c>
     </row>
@@ -8301,7 +8301,7 @@
       </c>
       <c r="V102" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11517.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11517.webp</t>
         </is>
       </c>
     </row>
@@ -8455,7 +8455,7 @@
       </c>
       <c r="V104" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11594.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11594.webp</t>
         </is>
       </c>
     </row>
@@ -8532,7 +8532,7 @@
       </c>
       <c r="V105" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11622.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11622.webp</t>
         </is>
       </c>
     </row>
@@ -8686,7 +8686,7 @@
       </c>
       <c r="V107" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11678.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11678.jpg</t>
         </is>
       </c>
     </row>
@@ -8840,7 +8840,7 @@
       </c>
       <c r="V109" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11800.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11800.webp</t>
         </is>
       </c>
     </row>
@@ -8917,7 +8917,7 @@
       </c>
       <c r="V110" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11809.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11809.jpg</t>
         </is>
       </c>
     </row>
@@ -8994,7 +8994,7 @@
       </c>
       <c r="V111" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11815.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11815.webp</t>
         </is>
       </c>
     </row>
@@ -9071,7 +9071,7 @@
       </c>
       <c r="V112" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11819.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11819.webp</t>
         </is>
       </c>
     </row>
@@ -9225,7 +9225,7 @@
       </c>
       <c r="V114" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11868.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11868.webp</t>
         </is>
       </c>
     </row>
@@ -9302,7 +9302,7 @@
       </c>
       <c r="V115" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11870.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11870.webp</t>
         </is>
       </c>
     </row>
@@ -9379,7 +9379,7 @@
       </c>
       <c r="V116" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11871.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11871.webp</t>
         </is>
       </c>
     </row>
@@ -9456,7 +9456,7 @@
       </c>
       <c r="V117" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11880.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11880.webp</t>
         </is>
       </c>
     </row>
@@ -9533,7 +9533,7 @@
       </c>
       <c r="V118" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11906.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11906.webp</t>
         </is>
       </c>
     </row>
@@ -9610,7 +9610,7 @@
       </c>
       <c r="V119" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11920.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11920.webp</t>
         </is>
       </c>
     </row>
@@ -9841,7 +9841,7 @@
       </c>
       <c r="V122" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11971.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11971.webp</t>
         </is>
       </c>
     </row>
@@ -9995,7 +9995,7 @@
       </c>
       <c r="V124" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/10276.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/10276.webp</t>
         </is>
       </c>
     </row>
@@ -10072,7 +10072,7 @@
       </c>
       <c r="V125" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/10504.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/10504.webp</t>
         </is>
       </c>
     </row>
@@ -10149,7 +10149,7 @@
       </c>
       <c r="V126" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/10982.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/10982.webp</t>
         </is>
       </c>
     </row>
@@ -10226,7 +10226,7 @@
       </c>
       <c r="V127" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11127.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11127.webp</t>
         </is>
       </c>
     </row>
@@ -10303,7 +10303,7 @@
       </c>
       <c r="V128" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11490.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11490.webp</t>
         </is>
       </c>
     </row>
@@ -10380,7 +10380,7 @@
       </c>
       <c r="V129" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11505.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11505.webp</t>
         </is>
       </c>
     </row>
@@ -10534,7 +10534,7 @@
       </c>
       <c r="V131" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11555.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11555.webp</t>
         </is>
       </c>
     </row>
@@ -10611,7 +10611,7 @@
       </c>
       <c r="V132" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11691.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11691.webp</t>
         </is>
       </c>
     </row>
@@ -10688,7 +10688,7 @@
       </c>
       <c r="V133" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11704.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11704.webp</t>
         </is>
       </c>
     </row>
@@ -10765,7 +10765,7 @@
       </c>
       <c r="V134" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11719.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11719.webp</t>
         </is>
       </c>
     </row>
@@ -10842,7 +10842,7 @@
       </c>
       <c r="V135" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11726.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11726.webp</t>
         </is>
       </c>
     </row>
@@ -11073,7 +11073,7 @@
       </c>
       <c r="V138" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11754.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11754.jpg</t>
         </is>
       </c>
     </row>
@@ -11150,7 +11150,7 @@
       </c>
       <c r="V139" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11757.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11757.webp</t>
         </is>
       </c>
     </row>
@@ -11227,7 +11227,7 @@
       </c>
       <c r="V140" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11758.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11758.webp</t>
         </is>
       </c>
     </row>
@@ -11304,7 +11304,7 @@
       </c>
       <c r="V141" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11760.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11760.webp</t>
         </is>
       </c>
     </row>
@@ -11381,7 +11381,7 @@
       </c>
       <c r="V142" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11762.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11762.webp</t>
         </is>
       </c>
     </row>
@@ -11458,7 +11458,7 @@
       </c>
       <c r="V143" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11763.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11763.webp</t>
         </is>
       </c>
     </row>
@@ -11612,7 +11612,7 @@
       </c>
       <c r="V145" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11767.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11767.webp</t>
         </is>
       </c>
     </row>
@@ -11689,7 +11689,7 @@
       </c>
       <c r="V146" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11769.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11769.webp</t>
         </is>
       </c>
     </row>
@@ -11766,7 +11766,7 @@
       </c>
       <c r="V147" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11771.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11771.webp</t>
         </is>
       </c>
     </row>
@@ -11843,7 +11843,7 @@
       </c>
       <c r="V148" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11772.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11772.webp</t>
         </is>
       </c>
     </row>
@@ -11920,7 +11920,7 @@
       </c>
       <c r="V149" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11774.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11774.webp</t>
         </is>
       </c>
     </row>
@@ -12074,7 +12074,7 @@
       </c>
       <c r="V151" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11777.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11777.webp</t>
         </is>
       </c>
     </row>
@@ -12151,7 +12151,7 @@
       </c>
       <c r="V152" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11778.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11778.webp</t>
         </is>
       </c>
     </row>
@@ -12305,7 +12305,7 @@
       </c>
       <c r="V154" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11780.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11780.webp</t>
         </is>
       </c>
     </row>
@@ -12382,7 +12382,7 @@
       </c>
       <c r="V155" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11781.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11781.webp</t>
         </is>
       </c>
     </row>
@@ -12459,7 +12459,7 @@
       </c>
       <c r="V156" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11782.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11782.webp</t>
         </is>
       </c>
     </row>
@@ -12536,7 +12536,7 @@
       </c>
       <c r="V157" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11783.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11783.webp</t>
         </is>
       </c>
     </row>
@@ -12613,7 +12613,7 @@
       </c>
       <c r="V158" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11784.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11784.webp</t>
         </is>
       </c>
     </row>
@@ -12767,7 +12767,7 @@
       </c>
       <c r="V160" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11787.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11787.webp</t>
         </is>
       </c>
     </row>
@@ -12844,7 +12844,7 @@
       </c>
       <c r="V161" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11789.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11789.webp</t>
         </is>
       </c>
     </row>
@@ -12921,7 +12921,7 @@
       </c>
       <c r="V162" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11790.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11790.webp</t>
         </is>
       </c>
     </row>
@@ -12998,7 +12998,7 @@
       </c>
       <c r="V163" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11791.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11791.webp</t>
         </is>
       </c>
     </row>
@@ -13152,7 +13152,7 @@
       </c>
       <c r="V165" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11794.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11794.webp</t>
         </is>
       </c>
     </row>
@@ -13229,7 +13229,7 @@
       </c>
       <c r="V166" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11795.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11795.webp</t>
         </is>
       </c>
     </row>
@@ -13383,7 +13383,7 @@
       </c>
       <c r="V168" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11952.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11952.webp</t>
         </is>
       </c>
     </row>
@@ -13460,7 +13460,7 @@
       </c>
       <c r="V169" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11953.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11953.webp</t>
         </is>
       </c>
     </row>
@@ -13614,7 +13614,7 @@
       </c>
       <c r="V171" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11972.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11972.webp</t>
         </is>
       </c>
     </row>
@@ -13691,7 +13691,7 @@
       </c>
       <c r="V172" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/12093.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/12093.webp</t>
         </is>
       </c>
     </row>
@@ -13768,7 +13768,7 @@
       </c>
       <c r="V173" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/10097.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/10097.png</t>
         </is>
       </c>
     </row>
@@ -13845,7 +13845,7 @@
       </c>
       <c r="V174" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/10883.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/10883.webp</t>
         </is>
       </c>
     </row>
@@ -13922,7 +13922,7 @@
       </c>
       <c r="V175" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11094.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11094.webp</t>
         </is>
       </c>
     </row>
@@ -13999,7 +13999,7 @@
       </c>
       <c r="V176" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11104.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11104.webp</t>
         </is>
       </c>
     </row>
@@ -14076,7 +14076,7 @@
       </c>
       <c r="V177" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11446.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11446.webp</t>
         </is>
       </c>
     </row>
@@ -14153,7 +14153,7 @@
       </c>
       <c r="V178" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11447.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11447.webp</t>
         </is>
       </c>
     </row>
@@ -14230,7 +14230,7 @@
       </c>
       <c r="V179" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11479.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11479.webp</t>
         </is>
       </c>
     </row>
@@ -14307,7 +14307,7 @@
       </c>
       <c r="V180" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11483.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11483.webp</t>
         </is>
       </c>
     </row>
@@ -14384,7 +14384,7 @@
       </c>
       <c r="V181" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11508.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11508.webp</t>
         </is>
       </c>
     </row>
@@ -14461,7 +14461,7 @@
       </c>
       <c r="V182" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11509.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11509.webp</t>
         </is>
       </c>
     </row>
@@ -14615,7 +14615,7 @@
       </c>
       <c r="V184" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11641.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11641.webp</t>
         </is>
       </c>
     </row>
@@ -14692,7 +14692,7 @@
       </c>
       <c r="V185" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11662.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11662.png</t>
         </is>
       </c>
     </row>
@@ -14769,7 +14769,7 @@
       </c>
       <c r="V186" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11693.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11693.png</t>
         </is>
       </c>
     </row>
@@ -14923,7 +14923,7 @@
       </c>
       <c r="V188" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11713.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11713.webp</t>
         </is>
       </c>
     </row>
@@ -15077,7 +15077,7 @@
       </c>
       <c r="V190" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11728.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11728.webp</t>
         </is>
       </c>
     </row>
@@ -15154,7 +15154,7 @@
       </c>
       <c r="V191" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11730.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11730.webp</t>
         </is>
       </c>
     </row>
@@ -15231,7 +15231,7 @@
       </c>
       <c r="V192" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11828.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11828.webp</t>
         </is>
       </c>
     </row>
@@ -15308,7 +15308,7 @@
       </c>
       <c r="V193" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11836.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11836.png</t>
         </is>
       </c>
     </row>
@@ -15385,7 +15385,7 @@
       </c>
       <c r="V194" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11929.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11929.webp</t>
         </is>
       </c>
     </row>
@@ -15462,7 +15462,7 @@
       </c>
       <c r="V195" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11943.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11943.png</t>
         </is>
       </c>
     </row>
@@ -15616,7 +15616,7 @@
       </c>
       <c r="V197" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/12035.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/12035.webp</t>
         </is>
       </c>
     </row>
@@ -15770,7 +15770,7 @@
       </c>
       <c r="V199" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/12054.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/12054.jpg</t>
         </is>
       </c>
     </row>
@@ -15847,7 +15847,7 @@
       </c>
       <c r="V200" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/12151.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/12151.webp</t>
         </is>
       </c>
     </row>
@@ -15924,7 +15924,7 @@
       </c>
       <c r="V201" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/10831.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/10831.webp</t>
         </is>
       </c>
     </row>
@@ -16001,7 +16001,7 @@
       </c>
       <c r="V202" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11491.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11491.webp</t>
         </is>
       </c>
     </row>
@@ -16078,7 +16078,7 @@
       </c>
       <c r="V203" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11515.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11515.webp</t>
         </is>
       </c>
     </row>
@@ -16155,7 +16155,7 @@
       </c>
       <c r="V204" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11528.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11528.webp</t>
         </is>
       </c>
     </row>
@@ -16232,7 +16232,7 @@
       </c>
       <c r="V205" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11535.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11535.webp</t>
         </is>
       </c>
     </row>
@@ -16309,7 +16309,7 @@
       </c>
       <c r="V206" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11536.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11536.jpg</t>
         </is>
       </c>
     </row>
@@ -16386,7 +16386,7 @@
       </c>
       <c r="V207" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11610.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11610.webp</t>
         </is>
       </c>
     </row>
@@ -16463,7 +16463,7 @@
       </c>
       <c r="V208" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11617.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11617.webp</t>
         </is>
       </c>
     </row>
@@ -16540,7 +16540,7 @@
       </c>
       <c r="V209" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11651.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11651.webp</t>
         </is>
       </c>
     </row>
@@ -16771,7 +16771,7 @@
       </c>
       <c r="V212" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11687.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11687.webp</t>
         </is>
       </c>
     </row>
@@ -16848,7 +16848,7 @@
       </c>
       <c r="V213" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11731.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11731.webp</t>
         </is>
       </c>
     </row>
@@ -16925,7 +16925,7 @@
       </c>
       <c r="V214" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11732.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11732.jpg</t>
         </is>
       </c>
     </row>
@@ -17233,7 +17233,7 @@
       </c>
       <c r="V218" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11738.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11738.webp</t>
         </is>
       </c>
     </row>
@@ -17310,7 +17310,7 @@
       </c>
       <c r="V219" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11741.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11741.webp</t>
         </is>
       </c>
     </row>
@@ -17387,7 +17387,7 @@
       </c>
       <c r="V220" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11743.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11743.webp</t>
         </is>
       </c>
     </row>
@@ -17464,7 +17464,7 @@
       </c>
       <c r="V221" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11744.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11744.png</t>
         </is>
       </c>
     </row>
@@ -17541,7 +17541,7 @@
       </c>
       <c r="V222" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11745.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11745.webp</t>
         </is>
       </c>
     </row>
@@ -17695,7 +17695,7 @@
       </c>
       <c r="V224" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11748.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11748.webp</t>
         </is>
       </c>
     </row>
@@ -17772,7 +17772,7 @@
       </c>
       <c r="V225" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11749.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11749.webp</t>
         </is>
       </c>
     </row>
@@ -17849,7 +17849,7 @@
       </c>
       <c r="V226" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11751.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11751.webp</t>
         </is>
       </c>
     </row>
@@ -17926,7 +17926,7 @@
       </c>
       <c r="V227" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11752.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11752.webp</t>
         </is>
       </c>
     </row>
@@ -18003,7 +18003,7 @@
       </c>
       <c r="V228" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11804.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11804.webp</t>
         </is>
       </c>
     </row>
@@ -18080,7 +18080,7 @@
       </c>
       <c r="V229" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11911.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11911.webp</t>
         </is>
       </c>
     </row>
@@ -18234,7 +18234,7 @@
       </c>
       <c r="V231" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11957.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11957.jpg</t>
         </is>
       </c>
     </row>
@@ -18388,7 +18388,7 @@
       </c>
       <c r="V233" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11959.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11959.webp</t>
         </is>
       </c>
     </row>
@@ -18542,7 +18542,7 @@
       </c>
       <c r="V235" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11961.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11961.webp</t>
         </is>
       </c>
     </row>
@@ -18696,7 +18696,7 @@
       </c>
       <c r="V237" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/12002.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/12002.webp</t>
         </is>
       </c>
     </row>
@@ -18773,7 +18773,7 @@
       </c>
       <c r="V238" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/12077.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/12077.webp</t>
         </is>
       </c>
     </row>
@@ -18850,7 +18850,7 @@
       </c>
       <c r="V239" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/12084.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/12084.webp</t>
         </is>
       </c>
     </row>
@@ -18927,7 +18927,7 @@
       </c>
       <c r="V240" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/12101.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/12101.jpg</t>
         </is>
       </c>
     </row>
@@ -19004,7 +19004,7 @@
       </c>
       <c r="V241" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/12102.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/12102.webp</t>
         </is>
       </c>
     </row>
@@ -19081,7 +19081,7 @@
       </c>
       <c r="V242" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/10449.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/10449.webp</t>
         </is>
       </c>
     </row>
@@ -19158,7 +19158,7 @@
       </c>
       <c r="V243" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/10988.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/10988.webp</t>
         </is>
       </c>
     </row>
@@ -19235,7 +19235,7 @@
       </c>
       <c r="V244" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/11184.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/11184.webp</t>
         </is>
       </c>
     </row>
@@ -19312,7 +19312,7 @@
       </c>
       <c r="V245" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/11518.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/11518.jpg</t>
         </is>
       </c>
     </row>
@@ -19389,7 +19389,7 @@
       </c>
       <c r="V246" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/11519.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/11519.webp</t>
         </is>
       </c>
     </row>
@@ -19466,7 +19466,7 @@
       </c>
       <c r="V247" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/11645.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/11645.webp</t>
         </is>
       </c>
     </row>
@@ -19543,7 +19543,7 @@
       </c>
       <c r="V248" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/11646.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/11646.webp</t>
         </is>
       </c>
     </row>
@@ -19620,7 +19620,7 @@
       </c>
       <c r="V249" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/11698.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/11698.webp</t>
         </is>
       </c>
     </row>
@@ -19697,7 +19697,7 @@
       </c>
       <c r="V250" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/11705.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/11705.webp</t>
         </is>
       </c>
     </row>
@@ -19774,7 +19774,7 @@
       </c>
       <c r="V251" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/11706.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/11706.webp</t>
         </is>
       </c>
     </row>
@@ -19851,7 +19851,7 @@
       </c>
       <c r="V252" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/11707.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/11707.webp</t>
         </is>
       </c>
     </row>
@@ -19928,7 +19928,7 @@
       </c>
       <c r="V253" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/11865.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/11865.webp</t>
         </is>
       </c>
     </row>
@@ -20005,7 +20005,7 @@
       </c>
       <c r="V254" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10058.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10058.webp</t>
         </is>
       </c>
     </row>
@@ -20082,7 +20082,7 @@
       </c>
       <c r="V255" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10061.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10061.webp</t>
         </is>
       </c>
     </row>
@@ -20159,7 +20159,7 @@
       </c>
       <c r="V256" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10102.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10102.webp</t>
         </is>
       </c>
     </row>
@@ -20236,7 +20236,7 @@
       </c>
       <c r="V257" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10171.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10171.webp</t>
         </is>
       </c>
     </row>
@@ -20313,7 +20313,7 @@
       </c>
       <c r="V258" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10256.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10256.webp</t>
         </is>
       </c>
     </row>
@@ -20390,7 +20390,7 @@
       </c>
       <c r="V259" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10264.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10264.webp</t>
         </is>
       </c>
     </row>
@@ -20467,7 +20467,7 @@
       </c>
       <c r="V260" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10306.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10306.jpg</t>
         </is>
       </c>
     </row>
@@ -20621,7 +20621,7 @@
       </c>
       <c r="V262" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10550.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10550.webp</t>
         </is>
       </c>
     </row>
@@ -20698,7 +20698,7 @@
       </c>
       <c r="V263" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10720.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10720.png</t>
         </is>
       </c>
     </row>
@@ -20775,7 +20775,7 @@
       </c>
       <c r="V264" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10887.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10887.webp</t>
         </is>
       </c>
     </row>
@@ -20852,7 +20852,7 @@
       </c>
       <c r="V265" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10902.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10902.webp</t>
         </is>
       </c>
     </row>
@@ -20929,7 +20929,7 @@
       </c>
       <c r="V266" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10967.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10967.webp</t>
         </is>
       </c>
     </row>
@@ -21006,7 +21006,7 @@
       </c>
       <c r="V267" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11029.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11029.webp</t>
         </is>
       </c>
     </row>
@@ -21160,7 +21160,7 @@
       </c>
       <c r="V269" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11168.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11168.webp</t>
         </is>
       </c>
     </row>
@@ -21237,7 +21237,7 @@
       </c>
       <c r="V270" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11170.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11170.webp</t>
         </is>
       </c>
     </row>
@@ -21314,7 +21314,7 @@
       </c>
       <c r="V271" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11237.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11237.webp</t>
         </is>
       </c>
     </row>
@@ -21391,7 +21391,7 @@
       </c>
       <c r="V272" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11382.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11382.webp</t>
         </is>
       </c>
     </row>
@@ -21468,7 +21468,7 @@
       </c>
       <c r="V273" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11466.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11466.webp</t>
         </is>
       </c>
     </row>
@@ -21545,7 +21545,7 @@
       </c>
       <c r="V274" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11468.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11468.webp</t>
         </is>
       </c>
     </row>
@@ -21622,7 +21622,7 @@
       </c>
       <c r="V275" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11473.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11473.webp</t>
         </is>
       </c>
     </row>
@@ -21699,7 +21699,7 @@
       </c>
       <c r="V276" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11487.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11487.png</t>
         </is>
       </c>
     </row>
@@ -21853,7 +21853,7 @@
       </c>
       <c r="V278" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11496.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11496.webp</t>
         </is>
       </c>
     </row>
@@ -21930,7 +21930,7 @@
       </c>
       <c r="V279" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11497.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11497.webp</t>
         </is>
       </c>
     </row>
@@ -22007,7 +22007,7 @@
       </c>
       <c r="V280" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11499.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11499.webp</t>
         </is>
       </c>
     </row>
@@ -22084,7 +22084,7 @@
       </c>
       <c r="V281" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11500.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11500.webp</t>
         </is>
       </c>
     </row>
@@ -22161,7 +22161,7 @@
       </c>
       <c r="V282" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11502.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11502.webp</t>
         </is>
       </c>
     </row>
@@ -22238,7 +22238,7 @@
       </c>
       <c r="V283" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11523.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11523.webp</t>
         </is>
       </c>
     </row>
@@ -22315,7 +22315,7 @@
       </c>
       <c r="V284" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11563.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11563.webp</t>
         </is>
       </c>
     </row>
@@ -22392,7 +22392,7 @@
       </c>
       <c r="V285" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11565.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11565.webp</t>
         </is>
       </c>
     </row>
@@ -22469,7 +22469,7 @@
       </c>
       <c r="V286" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11567.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11567.webp</t>
         </is>
       </c>
     </row>
@@ -22546,7 +22546,7 @@
       </c>
       <c r="V287" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11568.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11568.webp</t>
         </is>
       </c>
     </row>
@@ -22623,7 +22623,7 @@
       </c>
       <c r="V288" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11569.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11569.webp</t>
         </is>
       </c>
     </row>
@@ -22700,7 +22700,7 @@
       </c>
       <c r="V289" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11570.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11570.webp</t>
         </is>
       </c>
     </row>
@@ -22777,7 +22777,7 @@
       </c>
       <c r="V290" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11571.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11571.jpg</t>
         </is>
       </c>
     </row>
@@ -22854,7 +22854,7 @@
       </c>
       <c r="V291" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11572.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11572.webp</t>
         </is>
       </c>
     </row>
@@ -22931,7 +22931,7 @@
       </c>
       <c r="V292" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11573.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11573.webp</t>
         </is>
       </c>
     </row>
@@ -23008,7 +23008,7 @@
       </c>
       <c r="V293" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11584.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11584.webp</t>
         </is>
       </c>
     </row>
@@ -23085,7 +23085,7 @@
       </c>
       <c r="V294" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11586.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11586.webp</t>
         </is>
       </c>
     </row>
@@ -23162,7 +23162,7 @@
       </c>
       <c r="V295" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11588.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11588.webp</t>
         </is>
       </c>
     </row>
@@ -23239,7 +23239,7 @@
       </c>
       <c r="V296" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11592.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11592.webp</t>
         </is>
       </c>
     </row>
@@ -23316,7 +23316,7 @@
       </c>
       <c r="V297" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11602.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11602.webp</t>
         </is>
       </c>
     </row>
@@ -23393,7 +23393,7 @@
       </c>
       <c r="V298" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11607.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11607.webp</t>
         </is>
       </c>
     </row>
@@ -23470,7 +23470,7 @@
       </c>
       <c r="V299" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11608.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11608.webp</t>
         </is>
       </c>
     </row>
@@ -23547,7 +23547,7 @@
       </c>
       <c r="V300" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11629.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11629.webp</t>
         </is>
       </c>
     </row>
@@ -23624,7 +23624,7 @@
       </c>
       <c r="V301" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11630.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11630.webp</t>
         </is>
       </c>
     </row>
@@ -23701,7 +23701,7 @@
       </c>
       <c r="V302" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11642.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11642.webp</t>
         </is>
       </c>
     </row>
@@ -23778,7 +23778,7 @@
       </c>
       <c r="V303" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11643.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11643.webp</t>
         </is>
       </c>
     </row>
@@ -23855,7 +23855,7 @@
       </c>
       <c r="V304" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11647.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11647.webp</t>
         </is>
       </c>
     </row>
@@ -24009,7 +24009,7 @@
       </c>
       <c r="V306" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11717.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11717.webp</t>
         </is>
       </c>
     </row>
@@ -24086,7 +24086,7 @@
       </c>
       <c r="V307" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11806.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11806.webp</t>
         </is>
       </c>
     </row>
@@ -24163,7 +24163,7 @@
       </c>
       <c r="V308" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11818.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11818.webp</t>
         </is>
       </c>
     </row>
@@ -24240,7 +24240,7 @@
       </c>
       <c r="V309" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11822.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11822.webp</t>
         </is>
       </c>
     </row>
@@ -24317,7 +24317,7 @@
       </c>
       <c r="V310" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11830.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11830.webp</t>
         </is>
       </c>
     </row>
@@ -24394,7 +24394,7 @@
       </c>
       <c r="V311" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11833.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11833.webp</t>
         </is>
       </c>
     </row>
@@ -24471,7 +24471,7 @@
       </c>
       <c r="V312" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11834.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11834.webp</t>
         </is>
       </c>
     </row>
@@ -24548,7 +24548,7 @@
       </c>
       <c r="V313" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11838.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11838.webp</t>
         </is>
       </c>
     </row>
@@ -24702,7 +24702,7 @@
       </c>
       <c r="V315" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11840.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11840.webp</t>
         </is>
       </c>
     </row>
@@ -24856,7 +24856,7 @@
       </c>
       <c r="V317" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11844.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11844.webp</t>
         </is>
       </c>
     </row>
@@ -24933,7 +24933,7 @@
       </c>
       <c r="V318" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11845.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11845.webp</t>
         </is>
       </c>
     </row>
@@ -25010,7 +25010,7 @@
       </c>
       <c r="V319" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11863.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11863.webp</t>
         </is>
       </c>
     </row>
@@ -25241,7 +25241,7 @@
       </c>
       <c r="V322" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11875.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11875.webp</t>
         </is>
       </c>
     </row>
@@ -25318,7 +25318,7 @@
       </c>
       <c r="V323" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11877.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11877.webp</t>
         </is>
       </c>
     </row>
@@ -25472,7 +25472,7 @@
       </c>
       <c r="V325" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11909.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11909.webp</t>
         </is>
       </c>
     </row>
@@ -25549,7 +25549,7 @@
       </c>
       <c r="V326" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11910.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11910.webp</t>
         </is>
       </c>
     </row>
@@ -25626,7 +25626,7 @@
       </c>
       <c r="V327" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11913.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11913.webp</t>
         </is>
       </c>
     </row>
@@ -25703,7 +25703,7 @@
       </c>
       <c r="V328" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11931.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11931.webp</t>
         </is>
       </c>
     </row>
@@ -25780,7 +25780,7 @@
       </c>
       <c r="V329" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12004.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12004.png</t>
         </is>
       </c>
     </row>
@@ -25857,7 +25857,7 @@
       </c>
       <c r="V330" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12006.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12006.webp</t>
         </is>
       </c>
     </row>
@@ -25934,7 +25934,7 @@
       </c>
       <c r="V331" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12008.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12008.webp</t>
         </is>
       </c>
     </row>
@@ -26011,7 +26011,7 @@
       </c>
       <c r="V332" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12010.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12010.webp</t>
         </is>
       </c>
     </row>
@@ -26088,7 +26088,7 @@
       </c>
       <c r="V333" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12011.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12011.webp</t>
         </is>
       </c>
     </row>
@@ -26165,7 +26165,7 @@
       </c>
       <c r="V334" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12019.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12019.webp</t>
         </is>
       </c>
     </row>
@@ -26319,7 +26319,7 @@
       </c>
       <c r="V336" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12031.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12031.webp</t>
         </is>
       </c>
     </row>
@@ -26473,7 +26473,7 @@
       </c>
       <c r="V338" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12098.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12098.webp</t>
         </is>
       </c>
     </row>
@@ -26550,7 +26550,7 @@
       </c>
       <c r="V339" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12104.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12104.webp</t>
         </is>
       </c>
     </row>
@@ -26627,7 +26627,7 @@
       </c>
       <c r="V340" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12105.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12105.webp</t>
         </is>
       </c>
     </row>
@@ -26704,7 +26704,7 @@
       </c>
       <c r="V341" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12106.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12106.webp</t>
         </is>
       </c>
     </row>
@@ -26781,7 +26781,7 @@
       </c>
       <c r="V342" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12107.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12107.webp</t>
         </is>
       </c>
     </row>
@@ -26858,7 +26858,7 @@
       </c>
       <c r="V343" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12108.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12108.webp</t>
         </is>
       </c>
     </row>
@@ -27012,7 +27012,7 @@
       </c>
       <c r="V345" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12096.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12096.webp</t>
         </is>
       </c>
     </row>
@@ -27166,7 +27166,7 @@
       </c>
       <c r="V347" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12119.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12119.webp</t>
         </is>
       </c>
     </row>
@@ -27397,7 +27397,7 @@
       </c>
       <c r="V350" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12146.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12146.webp</t>
         </is>
       </c>
     </row>
@@ -27474,7 +27474,7 @@
       </c>
       <c r="V351" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12147.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12147.webp</t>
         </is>
       </c>
     </row>
@@ -27551,7 +27551,7 @@
       </c>
       <c r="V352" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12148.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12148.webp</t>
         </is>
       </c>
     </row>
@@ -27628,7 +27628,7 @@
       </c>
       <c r="V353" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12160.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12160.webp</t>
         </is>
       </c>
     </row>
@@ -27705,7 +27705,7 @@
       </c>
       <c r="V354" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12161.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12161.webp</t>
         </is>
       </c>
     </row>
@@ -27782,7 +27782,7 @@
       </c>
       <c r="V355" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12162.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12162.webp</t>
         </is>
       </c>
     </row>
@@ -27859,7 +27859,7 @@
       </c>
       <c r="V356" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12164.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12164.webp</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
re-download sem CDN de loja
</commit_message>
<xml_diff>
--- a/PLANILHA-FOTOS-NOVAS-355.xlsx
+++ b/PLANILHA-FOTOS-NOVAS-355.xlsx
@@ -678,7 +678,7 @@
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/adocantes-naturais/11511.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/adocantes-naturais/11511.jpg</t>
         </is>
       </c>
     </row>
@@ -909,7 +909,7 @@
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/adocantes-naturais/12027.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/adocantes-naturais/12027.png</t>
         </is>
       </c>
     </row>
@@ -1063,7 +1063,7 @@
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/adocantes-naturais/12174.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/adocantes-naturais/12174.png</t>
         </is>
       </c>
     </row>
@@ -1140,7 +1140,7 @@
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10043.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10043.jpg</t>
         </is>
       </c>
     </row>
@@ -1217,7 +1217,7 @@
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10092.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10092.jpg</t>
         </is>
       </c>
     </row>
@@ -1294,7 +1294,7 @@
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10115.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10115.jpg</t>
         </is>
       </c>
     </row>
@@ -1371,7 +1371,7 @@
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10217.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10217.jpg</t>
         </is>
       </c>
     </row>
@@ -1525,7 +1525,7 @@
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10364.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10364.jpg</t>
         </is>
       </c>
     </row>
@@ -1602,7 +1602,7 @@
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10395.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10395.jpg</t>
         </is>
       </c>
     </row>
@@ -1679,7 +1679,7 @@
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10396.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10396.jpg</t>
         </is>
       </c>
     </row>
@@ -1756,7 +1756,7 @@
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10652.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10652.jpg</t>
         </is>
       </c>
     </row>
@@ -1833,7 +1833,7 @@
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10745.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10745.jpg</t>
         </is>
       </c>
     </row>
@@ -1987,7 +1987,7 @@
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10877.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10877.jpg</t>
         </is>
       </c>
     </row>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10900.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10900.jpg</t>
         </is>
       </c>
     </row>
@@ -2218,7 +2218,7 @@
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10910.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10910.jpg</t>
         </is>
       </c>
     </row>
@@ -2295,7 +2295,7 @@
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10914.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10914.jpg</t>
         </is>
       </c>
     </row>
@@ -2372,7 +2372,7 @@
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10915.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10915.jpg</t>
         </is>
       </c>
     </row>
@@ -2449,7 +2449,7 @@
       </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10946.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10946.jpg</t>
         </is>
       </c>
     </row>
@@ -2526,7 +2526,7 @@
       </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10957.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10957.jpg</t>
         </is>
       </c>
     </row>
@@ -2603,7 +2603,7 @@
       </c>
       <c r="V28" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10978.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10978.png</t>
         </is>
       </c>
     </row>
@@ -2680,7 +2680,7 @@
       </c>
       <c r="V29" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11005.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11005.jpg</t>
         </is>
       </c>
     </row>
@@ -2834,7 +2834,7 @@
       </c>
       <c r="V31" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11055.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11055.jpg</t>
         </is>
       </c>
     </row>
@@ -2911,7 +2911,7 @@
       </c>
       <c r="V32" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11059.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11059.jpg</t>
         </is>
       </c>
     </row>
@@ -2988,7 +2988,7 @@
       </c>
       <c r="V33" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11061.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11061.jpg</t>
         </is>
       </c>
     </row>
@@ -3065,7 +3065,7 @@
       </c>
       <c r="V34" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11062.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11062.jpg</t>
         </is>
       </c>
     </row>
@@ -3142,7 +3142,7 @@
       </c>
       <c r="V35" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11077.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11077.jpg</t>
         </is>
       </c>
     </row>
@@ -3373,7 +3373,7 @@
       </c>
       <c r="V38" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11110.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11110.jpg</t>
         </is>
       </c>
     </row>
@@ -3450,7 +3450,7 @@
       </c>
       <c r="V39" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11116.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11116.jpg</t>
         </is>
       </c>
     </row>
@@ -3758,7 +3758,7 @@
       </c>
       <c r="V43" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11125.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11125.jpg</t>
         </is>
       </c>
     </row>
@@ -3835,7 +3835,7 @@
       </c>
       <c r="V44" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11132.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11132.jpg</t>
         </is>
       </c>
     </row>
@@ -3912,7 +3912,7 @@
       </c>
       <c r="V45" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11136.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11136.png</t>
         </is>
       </c>
     </row>
@@ -3989,7 +3989,7 @@
       </c>
       <c r="V46" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11137.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11137.jpg</t>
         </is>
       </c>
     </row>
@@ -4066,7 +4066,7 @@
       </c>
       <c r="V47" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11160.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11160.jpg</t>
         </is>
       </c>
     </row>
@@ -4143,7 +4143,7 @@
       </c>
       <c r="V48" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11175.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11175.jpg</t>
         </is>
       </c>
     </row>
@@ -4220,7 +4220,7 @@
       </c>
       <c r="V49" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11259.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11259.jpg</t>
         </is>
       </c>
     </row>
@@ -4374,7 +4374,7 @@
       </c>
       <c r="V51" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11325.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11325.jpg</t>
         </is>
       </c>
     </row>
@@ -4605,7 +4605,7 @@
       </c>
       <c r="V54" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11331.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11331.jpg</t>
         </is>
       </c>
     </row>
@@ -4682,7 +4682,7 @@
       </c>
       <c r="V55" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11332.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11332.jpg</t>
         </is>
       </c>
     </row>
@@ -4759,7 +4759,7 @@
       </c>
       <c r="V56" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11334.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11334.png</t>
         </is>
       </c>
     </row>
@@ -4913,7 +4913,7 @@
       </c>
       <c r="V58" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11337.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11337.png</t>
         </is>
       </c>
     </row>
@@ -4990,7 +4990,7 @@
       </c>
       <c r="V59" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11338.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11338.png</t>
         </is>
       </c>
     </row>
@@ -5144,7 +5144,7 @@
       </c>
       <c r="V61" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11340.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11340.jpg</t>
         </is>
       </c>
     </row>
@@ -5221,7 +5221,7 @@
       </c>
       <c r="V62" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11341.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11341.jpg</t>
         </is>
       </c>
     </row>
@@ -5298,7 +5298,7 @@
       </c>
       <c r="V63" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11342.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11342.jpg</t>
         </is>
       </c>
     </row>
@@ -5452,7 +5452,7 @@
       </c>
       <c r="V65" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11401.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11401.jpg</t>
         </is>
       </c>
     </row>
@@ -5683,7 +5683,7 @@
       </c>
       <c r="V68" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/12052.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/12052.jpg</t>
         </is>
       </c>
     </row>
@@ -5760,7 +5760,7 @@
       </c>
       <c r="V69" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/12091.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/12091.jpg</t>
         </is>
       </c>
     </row>
@@ -6145,7 +6145,7 @@
       </c>
       <c r="V74" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/10037.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/10037.jpg</t>
         </is>
       </c>
     </row>
@@ -6376,7 +6376,7 @@
       </c>
       <c r="V77" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/10073.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/10073.png</t>
         </is>
       </c>
     </row>
@@ -6607,7 +6607,7 @@
       </c>
       <c r="V80" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11803.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11803.webp</t>
         </is>
       </c>
     </row>
@@ -6684,7 +6684,7 @@
       </c>
       <c r="V81" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11848.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11848.png</t>
         </is>
       </c>
     </row>
@@ -6761,7 +6761,7 @@
       </c>
       <c r="V82" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11861.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11861.jpg</t>
         </is>
       </c>
     </row>
@@ -6838,7 +6838,7 @@
       </c>
       <c r="V83" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11902.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11902.png</t>
         </is>
       </c>
     </row>
@@ -6915,7 +6915,7 @@
       </c>
       <c r="V84" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11939.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11939.png</t>
         </is>
       </c>
     </row>
@@ -7069,7 +7069,7 @@
       </c>
       <c r="V86" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11998.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11998.jpg</t>
         </is>
       </c>
     </row>
@@ -7146,7 +7146,7 @@
       </c>
       <c r="V87" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/12039.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/12039.jpg</t>
         </is>
       </c>
     </row>
@@ -7300,7 +7300,7 @@
       </c>
       <c r="V89" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/12086.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/12086.jpg</t>
         </is>
       </c>
     </row>
@@ -7377,7 +7377,7 @@
       </c>
       <c r="V90" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/12072.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/12072.jpg</t>
         </is>
       </c>
     </row>
@@ -7454,7 +7454,7 @@
       </c>
       <c r="V91" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/10277.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/10277.jpg</t>
         </is>
       </c>
     </row>
@@ -7608,7 +7608,7 @@
       </c>
       <c r="V93" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/10873.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/10873.jpg</t>
         </is>
       </c>
     </row>
@@ -7685,7 +7685,7 @@
       </c>
       <c r="V94" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/11480.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/11480.jpg</t>
         </is>
       </c>
     </row>
@@ -7762,7 +7762,7 @@
       </c>
       <c r="V95" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/11895.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/11895.jpg</t>
         </is>
       </c>
     </row>
@@ -7839,7 +7839,7 @@
       </c>
       <c r="V96" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/11898.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/11898.png</t>
         </is>
       </c>
     </row>
@@ -8070,7 +8070,7 @@
       </c>
       <c r="V99" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/11951.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/11951.webp</t>
         </is>
       </c>
     </row>
@@ -8224,7 +8224,7 @@
       </c>
       <c r="V101" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/10944.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/10944.png</t>
         </is>
       </c>
     </row>
@@ -8301,7 +8301,7 @@
       </c>
       <c r="V102" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11517.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11517.png</t>
         </is>
       </c>
     </row>
@@ -8455,7 +8455,7 @@
       </c>
       <c r="V104" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11594.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11594.jpg</t>
         </is>
       </c>
     </row>
@@ -8840,7 +8840,7 @@
       </c>
       <c r="V109" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11800.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11800.jpg</t>
         </is>
       </c>
     </row>
@@ -8994,7 +8994,7 @@
       </c>
       <c r="V111" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11815.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11815.jpg</t>
         </is>
       </c>
     </row>
@@ -9071,7 +9071,7 @@
       </c>
       <c r="V112" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11819.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11819.jpg</t>
         </is>
       </c>
     </row>
@@ -9225,7 +9225,7 @@
       </c>
       <c r="V114" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11868.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11868.jpg</t>
         </is>
       </c>
     </row>
@@ -9456,7 +9456,7 @@
       </c>
       <c r="V117" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11880.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11880.jpg</t>
         </is>
       </c>
     </row>
@@ -9533,7 +9533,7 @@
       </c>
       <c r="V118" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11906.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11906.jpg</t>
         </is>
       </c>
     </row>
@@ -9610,7 +9610,7 @@
       </c>
       <c r="V119" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11920.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11920.jpg</t>
         </is>
       </c>
     </row>
@@ -9764,7 +9764,7 @@
       </c>
       <c r="V121" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11968.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11968.jpg</t>
         </is>
       </c>
     </row>
@@ -9841,7 +9841,7 @@
       </c>
       <c r="V122" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11971.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11971.png</t>
         </is>
       </c>
     </row>
@@ -9995,7 +9995,7 @@
       </c>
       <c r="V124" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/10276.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/10276.jpg</t>
         </is>
       </c>
     </row>
@@ -10072,7 +10072,7 @@
       </c>
       <c r="V125" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/10504.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/10504.jpg</t>
         </is>
       </c>
     </row>
@@ -10149,7 +10149,7 @@
       </c>
       <c r="V126" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/10982.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/10982.jpg</t>
         </is>
       </c>
     </row>
@@ -10226,7 +10226,7 @@
       </c>
       <c r="V127" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11127.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11127.jpg</t>
         </is>
       </c>
     </row>
@@ -10303,7 +10303,7 @@
       </c>
       <c r="V128" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11490.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11490.jpg</t>
         </is>
       </c>
     </row>
@@ -10380,7 +10380,7 @@
       </c>
       <c r="V129" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11505.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11505.jpg</t>
         </is>
       </c>
     </row>
@@ -10534,7 +10534,7 @@
       </c>
       <c r="V131" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11555.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11555.jpg</t>
         </is>
       </c>
     </row>
@@ -10611,7 +10611,7 @@
       </c>
       <c r="V132" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11691.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11691.jpg</t>
         </is>
       </c>
     </row>
@@ -10688,7 +10688,7 @@
       </c>
       <c r="V133" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11704.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11704.jpg</t>
         </is>
       </c>
     </row>
@@ -10765,7 +10765,7 @@
       </c>
       <c r="V134" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11719.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11719.png</t>
         </is>
       </c>
     </row>
@@ -10842,7 +10842,7 @@
       </c>
       <c r="V135" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11726.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11726.png</t>
         </is>
       </c>
     </row>
@@ -10919,7 +10919,7 @@
       </c>
       <c r="V136" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11750.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11750.png</t>
         </is>
       </c>
     </row>
@@ -11150,7 +11150,7 @@
       </c>
       <c r="V139" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11757.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11757.jpg</t>
         </is>
       </c>
     </row>
@@ -11227,7 +11227,7 @@
       </c>
       <c r="V140" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11758.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11758.jpg</t>
         </is>
       </c>
     </row>
@@ -11381,7 +11381,7 @@
       </c>
       <c r="V142" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11762.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11762.png</t>
         </is>
       </c>
     </row>
@@ -11458,7 +11458,7 @@
       </c>
       <c r="V143" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11763.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11763.png</t>
         </is>
       </c>
     </row>
@@ -11612,7 +11612,7 @@
       </c>
       <c r="V145" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11767.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11767.png</t>
         </is>
       </c>
     </row>
@@ -11689,7 +11689,7 @@
       </c>
       <c r="V146" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11769.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11769.jpg</t>
         </is>
       </c>
     </row>
@@ -11766,7 +11766,7 @@
       </c>
       <c r="V147" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11771.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11771.png</t>
         </is>
       </c>
     </row>
@@ -11843,7 +11843,7 @@
       </c>
       <c r="V148" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11772.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11772.jpg</t>
         </is>
       </c>
     </row>
@@ -11920,7 +11920,7 @@
       </c>
       <c r="V149" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11774.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11774.png</t>
         </is>
       </c>
     </row>
@@ -12074,7 +12074,7 @@
       </c>
       <c r="V151" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11777.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11777.jpg</t>
         </is>
       </c>
     </row>
@@ -12151,7 +12151,7 @@
       </c>
       <c r="V152" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11778.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11778.jpg</t>
         </is>
       </c>
     </row>
@@ -12305,7 +12305,7 @@
       </c>
       <c r="V154" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11780.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11780.jpg</t>
         </is>
       </c>
     </row>
@@ -12382,7 +12382,7 @@
       </c>
       <c r="V155" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11781.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11781.jpg</t>
         </is>
       </c>
     </row>
@@ -12459,7 +12459,7 @@
       </c>
       <c r="V156" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11782.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11782.jpg</t>
         </is>
       </c>
     </row>
@@ -12613,7 +12613,7 @@
       </c>
       <c r="V158" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11784.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11784.png</t>
         </is>
       </c>
     </row>
@@ -12767,7 +12767,7 @@
       </c>
       <c r="V160" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11787.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11787.jpg</t>
         </is>
       </c>
     </row>
@@ -12844,7 +12844,7 @@
       </c>
       <c r="V161" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11789.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11789.jpg</t>
         </is>
       </c>
     </row>
@@ -13152,7 +13152,7 @@
       </c>
       <c r="V165" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11794.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11794.jpg</t>
         </is>
       </c>
     </row>
@@ -13229,7 +13229,7 @@
       </c>
       <c r="V166" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11795.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11795.jpg</t>
         </is>
       </c>
     </row>
@@ -13306,7 +13306,7 @@
       </c>
       <c r="V167" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11796.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11796.png</t>
         </is>
       </c>
     </row>
@@ -13383,7 +13383,7 @@
       </c>
       <c r="V168" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11952.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11952.jpg</t>
         </is>
       </c>
     </row>
@@ -13614,7 +13614,7 @@
       </c>
       <c r="V171" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11972.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11972.png</t>
         </is>
       </c>
     </row>
@@ -13691,7 +13691,7 @@
       </c>
       <c r="V172" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/12093.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/12093.jpg</t>
         </is>
       </c>
     </row>
@@ -13845,7 +13845,7 @@
       </c>
       <c r="V174" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/10883.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/10883.jpg</t>
         </is>
       </c>
     </row>
@@ -13922,7 +13922,7 @@
       </c>
       <c r="V175" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11094.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11094.jpg</t>
         </is>
       </c>
     </row>
@@ -13999,7 +13999,7 @@
       </c>
       <c r="V176" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11104.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11104.jpg</t>
         </is>
       </c>
     </row>
@@ -14076,7 +14076,7 @@
       </c>
       <c r="V177" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11446.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11446.png</t>
         </is>
       </c>
     </row>
@@ -14153,7 +14153,7 @@
       </c>
       <c r="V178" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11447.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11447.png</t>
         </is>
       </c>
     </row>
@@ -14230,7 +14230,7 @@
       </c>
       <c r="V179" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11479.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11479.jpg</t>
         </is>
       </c>
     </row>
@@ -14307,7 +14307,7 @@
       </c>
       <c r="V180" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11483.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11483.jpg</t>
         </is>
       </c>
     </row>
@@ -14384,7 +14384,7 @@
       </c>
       <c r="V181" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11508.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11508.jpg</t>
         </is>
       </c>
     </row>
@@ -14461,7 +14461,7 @@
       </c>
       <c r="V182" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11509.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11509.png</t>
         </is>
       </c>
     </row>
@@ -14923,7 +14923,7 @@
       </c>
       <c r="V188" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11713.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11713.jpg</t>
         </is>
       </c>
     </row>
@@ -15077,7 +15077,7 @@
       </c>
       <c r="V190" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11728.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11728.jpg</t>
         </is>
       </c>
     </row>
@@ -15154,7 +15154,7 @@
       </c>
       <c r="V191" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11730.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11730.jpg</t>
         </is>
       </c>
     </row>
@@ -15231,7 +15231,7 @@
       </c>
       <c r="V192" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11828.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11828.jpg</t>
         </is>
       </c>
     </row>
@@ -15308,7 +15308,7 @@
       </c>
       <c r="V193" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11836.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11836.jpg</t>
         </is>
       </c>
     </row>
@@ -15385,7 +15385,7 @@
       </c>
       <c r="V194" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11929.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11929.jpg</t>
         </is>
       </c>
     </row>
@@ -15616,7 +15616,7 @@
       </c>
       <c r="V197" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/12035.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/12035.png</t>
         </is>
       </c>
     </row>
@@ -15847,7 +15847,7 @@
       </c>
       <c r="V200" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/12151.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/12151.jpg</t>
         </is>
       </c>
     </row>
@@ -15924,7 +15924,7 @@
       </c>
       <c r="V201" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/10831.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/10831.jpg</t>
         </is>
       </c>
     </row>
@@ -16001,7 +16001,7 @@
       </c>
       <c r="V202" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11491.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11491.jpg</t>
         </is>
       </c>
     </row>
@@ -16078,7 +16078,7 @@
       </c>
       <c r="V203" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11515.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11515.jpg</t>
         </is>
       </c>
     </row>
@@ -16232,7 +16232,7 @@
       </c>
       <c r="V205" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11535.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11535.jpg</t>
         </is>
       </c>
     </row>
@@ -16386,7 +16386,7 @@
       </c>
       <c r="V207" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11610.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11610.jpg</t>
         </is>
       </c>
     </row>
@@ -16463,7 +16463,7 @@
       </c>
       <c r="V208" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11617.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11617.jpg</t>
         </is>
       </c>
     </row>
@@ -16540,7 +16540,7 @@
       </c>
       <c r="V209" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11651.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11651.jpg</t>
         </is>
       </c>
     </row>
@@ -16694,7 +16694,7 @@
       </c>
       <c r="V211" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11686.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11686.png</t>
         </is>
       </c>
     </row>
@@ -16848,7 +16848,7 @@
       </c>
       <c r="V213" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11731.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11731.jpg</t>
         </is>
       </c>
     </row>
@@ -17233,7 +17233,7 @@
       </c>
       <c r="V218" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11738.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11738.jpg</t>
         </is>
       </c>
     </row>
@@ -17310,7 +17310,7 @@
       </c>
       <c r="V219" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11741.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11741.jpg</t>
         </is>
       </c>
     </row>
@@ -17464,7 +17464,7 @@
       </c>
       <c r="V221" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11744.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11744.jpg</t>
         </is>
       </c>
     </row>
@@ -17541,7 +17541,7 @@
       </c>
       <c r="V222" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11745.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11745.jpg</t>
         </is>
       </c>
     </row>
@@ -17772,7 +17772,7 @@
       </c>
       <c r="V225" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11749.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11749.jpg</t>
         </is>
       </c>
     </row>
@@ -17849,7 +17849,7 @@
       </c>
       <c r="V226" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11751.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11751.jpg</t>
         </is>
       </c>
     </row>
@@ -17926,7 +17926,7 @@
       </c>
       <c r="V227" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11752.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11752.jpg</t>
         </is>
       </c>
     </row>
@@ -18080,7 +18080,7 @@
       </c>
       <c r="V229" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11911.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11911.jpg</t>
         </is>
       </c>
     </row>
@@ -18157,7 +18157,7 @@
       </c>
       <c r="V230" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11912.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11912.jpg</t>
         </is>
       </c>
     </row>
@@ -18311,7 +18311,7 @@
       </c>
       <c r="V232" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11958.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11958.jpg</t>
         </is>
       </c>
     </row>
@@ -18773,7 +18773,7 @@
       </c>
       <c r="V238" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/12077.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/12077.jpg</t>
         </is>
       </c>
     </row>
@@ -19004,7 +19004,7 @@
       </c>
       <c r="V241" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/12102.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/12102.png</t>
         </is>
       </c>
     </row>
@@ -19081,7 +19081,7 @@
       </c>
       <c r="V242" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/10449.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/10449.jpg</t>
         </is>
       </c>
     </row>
@@ -19158,7 +19158,7 @@
       </c>
       <c r="V243" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/10988.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/10988.jpg</t>
         </is>
       </c>
     </row>
@@ -19235,7 +19235,7 @@
       </c>
       <c r="V244" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/11184.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/11184.jpg</t>
         </is>
       </c>
     </row>
@@ -19389,7 +19389,7 @@
       </c>
       <c r="V246" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/11519.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/11519.jpg</t>
         </is>
       </c>
     </row>
@@ -19466,7 +19466,7 @@
       </c>
       <c r="V247" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/11645.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/11645.jpg</t>
         </is>
       </c>
     </row>
@@ -19543,7 +19543,7 @@
       </c>
       <c r="V248" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/11646.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/11646.jpg</t>
         </is>
       </c>
     </row>
@@ -19697,7 +19697,7 @@
       </c>
       <c r="V250" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/11705.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/11705.jpg</t>
         </is>
       </c>
     </row>
@@ -19774,7 +19774,7 @@
       </c>
       <c r="V251" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/11706.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/11706.png</t>
         </is>
       </c>
     </row>
@@ -19851,7 +19851,7 @@
       </c>
       <c r="V252" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/11707.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/11707.jpg</t>
         </is>
       </c>
     </row>
@@ -19928,7 +19928,7 @@
       </c>
       <c r="V253" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/11865.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/11865.jpg</t>
         </is>
       </c>
     </row>
@@ -20005,7 +20005,7 @@
       </c>
       <c r="V254" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10058.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10058.jpg</t>
         </is>
       </c>
     </row>
@@ -20082,7 +20082,7 @@
       </c>
       <c r="V255" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10061.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10061.jpg</t>
         </is>
       </c>
     </row>
@@ -20236,7 +20236,7 @@
       </c>
       <c r="V257" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10171.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10171.jpg</t>
         </is>
       </c>
     </row>
@@ -20390,7 +20390,7 @@
       </c>
       <c r="V259" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10264.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10264.jpg</t>
         </is>
       </c>
     </row>
@@ -20544,7 +20544,7 @@
       </c>
       <c r="V261" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10308.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10308.jpg</t>
         </is>
       </c>
     </row>
@@ -20621,7 +20621,7 @@
       </c>
       <c r="V262" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10550.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10550.png</t>
         </is>
       </c>
     </row>
@@ -20698,7 +20698,7 @@
       </c>
       <c r="V263" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10720.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10720.jpg</t>
         </is>
       </c>
     </row>
@@ -20775,7 +20775,7 @@
       </c>
       <c r="V264" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10887.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10887.png</t>
         </is>
       </c>
     </row>
@@ -20852,7 +20852,7 @@
       </c>
       <c r="V265" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10902.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10902.png</t>
         </is>
       </c>
     </row>
@@ -20929,7 +20929,7 @@
       </c>
       <c r="V266" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10967.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10967.jpg</t>
         </is>
       </c>
     </row>
@@ -21160,7 +21160,7 @@
       </c>
       <c r="V269" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11168.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11168.jpg</t>
         </is>
       </c>
     </row>
@@ -21237,7 +21237,7 @@
       </c>
       <c r="V270" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11170.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11170.jpg</t>
         </is>
       </c>
     </row>
@@ -21314,7 +21314,7 @@
       </c>
       <c r="V271" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11237.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11237.png</t>
         </is>
       </c>
     </row>
@@ -21468,7 +21468,7 @@
       </c>
       <c r="V273" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11466.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11466.jpg</t>
         </is>
       </c>
     </row>
@@ -21622,7 +21622,7 @@
       </c>
       <c r="V275" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11473.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11473.jpg</t>
         </is>
       </c>
     </row>
@@ -21776,7 +21776,7 @@
       </c>
       <c r="V277" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11493.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11493.jpg</t>
         </is>
       </c>
     </row>
@@ -21853,7 +21853,7 @@
       </c>
       <c r="V278" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11496.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11496.jpg</t>
         </is>
       </c>
     </row>
@@ -21930,7 +21930,7 @@
       </c>
       <c r="V279" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11497.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11497.jpg</t>
         </is>
       </c>
     </row>
@@ -22084,7 +22084,7 @@
       </c>
       <c r="V281" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11500.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11500.jpg</t>
         </is>
       </c>
     </row>
@@ -22161,7 +22161,7 @@
       </c>
       <c r="V282" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11502.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11502.jpg</t>
         </is>
       </c>
     </row>
@@ -22238,7 +22238,7 @@
       </c>
       <c r="V283" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11523.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11523.jpg</t>
         </is>
       </c>
     </row>
@@ -22315,7 +22315,7 @@
       </c>
       <c r="V284" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11563.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11563.png</t>
         </is>
       </c>
     </row>
@@ -22392,7 +22392,7 @@
       </c>
       <c r="V285" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11565.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11565.jpg</t>
         </is>
       </c>
     </row>
@@ -22469,7 +22469,7 @@
       </c>
       <c r="V286" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11567.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11567.jpg</t>
         </is>
       </c>
     </row>
@@ -22623,7 +22623,7 @@
       </c>
       <c r="V288" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11569.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11569.jpg</t>
         </is>
       </c>
     </row>
@@ -22700,7 +22700,7 @@
       </c>
       <c r="V289" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11570.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11570.png</t>
         </is>
       </c>
     </row>
@@ -22931,7 +22931,7 @@
       </c>
       <c r="V292" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11573.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11573.jpg</t>
         </is>
       </c>
     </row>
@@ -23008,7 +23008,7 @@
       </c>
       <c r="V293" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11584.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11584.jpg</t>
         </is>
       </c>
     </row>
@@ -23085,7 +23085,7 @@
       </c>
       <c r="V294" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11586.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11586.jpg</t>
         </is>
       </c>
     </row>
@@ -23162,7 +23162,7 @@
       </c>
       <c r="V295" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11588.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11588.jpg</t>
         </is>
       </c>
     </row>
@@ -23239,7 +23239,7 @@
       </c>
       <c r="V296" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11592.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11592.jpg</t>
         </is>
       </c>
     </row>
@@ -23316,7 +23316,7 @@
       </c>
       <c r="V297" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11602.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11602.jpg</t>
         </is>
       </c>
     </row>
@@ -23393,7 +23393,7 @@
       </c>
       <c r="V298" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11607.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11607.jpg</t>
         </is>
       </c>
     </row>
@@ -23470,7 +23470,7 @@
       </c>
       <c r="V299" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11608.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11608.jpg</t>
         </is>
       </c>
     </row>
@@ -23547,7 +23547,7 @@
       </c>
       <c r="V300" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11629.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11629.jpg</t>
         </is>
       </c>
     </row>
@@ -23624,7 +23624,7 @@
       </c>
       <c r="V301" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11630.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11630.png</t>
         </is>
       </c>
     </row>
@@ -23701,7 +23701,7 @@
       </c>
       <c r="V302" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11642.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11642.png</t>
         </is>
       </c>
     </row>
@@ -23855,7 +23855,7 @@
       </c>
       <c r="V304" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11647.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11647.jpg</t>
         </is>
       </c>
     </row>
@@ -24009,7 +24009,7 @@
       </c>
       <c r="V306" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11717.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11717.jpg</t>
         </is>
       </c>
     </row>
@@ -24086,7 +24086,7 @@
       </c>
       <c r="V307" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11806.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11806.jpg</t>
         </is>
       </c>
     </row>
@@ -24163,7 +24163,7 @@
       </c>
       <c r="V308" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11818.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11818.jpg</t>
         </is>
       </c>
     </row>
@@ -24240,7 +24240,7 @@
       </c>
       <c r="V309" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11822.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11822.jpg</t>
         </is>
       </c>
     </row>
@@ -24317,7 +24317,7 @@
       </c>
       <c r="V310" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11830.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11830.jpg</t>
         </is>
       </c>
     </row>
@@ -24394,7 +24394,7 @@
       </c>
       <c r="V311" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11833.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11833.jpg</t>
         </is>
       </c>
     </row>
@@ -24471,7 +24471,7 @@
       </c>
       <c r="V312" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11834.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11834.png</t>
         </is>
       </c>
     </row>
@@ -24548,7 +24548,7 @@
       </c>
       <c r="V313" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11838.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11838.png</t>
         </is>
       </c>
     </row>
@@ -24702,7 +24702,7 @@
       </c>
       <c r="V315" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11840.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11840.jpg</t>
         </is>
       </c>
     </row>
@@ -24779,7 +24779,7 @@
       </c>
       <c r="V316" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11843.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11843.jpg</t>
         </is>
       </c>
     </row>
@@ -24856,7 +24856,7 @@
       </c>
       <c r="V317" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11844.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11844.jpg</t>
         </is>
       </c>
     </row>
@@ -24933,7 +24933,7 @@
       </c>
       <c r="V318" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11845.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11845.png</t>
         </is>
       </c>
     </row>
@@ -25010,7 +25010,7 @@
       </c>
       <c r="V319" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11863.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11863.jpg</t>
         </is>
       </c>
     </row>
@@ -25241,7 +25241,7 @@
       </c>
       <c r="V322" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11875.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11875.jpg</t>
         </is>
       </c>
     </row>
@@ -25318,7 +25318,7 @@
       </c>
       <c r="V323" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11877.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11877.jpg</t>
         </is>
       </c>
     </row>
@@ -25472,7 +25472,7 @@
       </c>
       <c r="V325" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11909.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11909.jpg</t>
         </is>
       </c>
     </row>
@@ -25549,7 +25549,7 @@
       </c>
       <c r="V326" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11910.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11910.png</t>
         </is>
       </c>
     </row>
@@ -25626,7 +25626,7 @@
       </c>
       <c r="V327" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11913.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11913.jpg</t>
         </is>
       </c>
     </row>
@@ -25703,7 +25703,7 @@
       </c>
       <c r="V328" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11931.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11931.png</t>
         </is>
       </c>
     </row>
@@ -25780,7 +25780,7 @@
       </c>
       <c r="V329" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12004.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12004.jpg</t>
         </is>
       </c>
     </row>
@@ -26088,7 +26088,7 @@
       </c>
       <c r="V333" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12011.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12011.jpg</t>
         </is>
       </c>
     </row>
@@ -26165,7 +26165,7 @@
       </c>
       <c r="V334" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12019.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12019.jpg</t>
         </is>
       </c>
     </row>
@@ -26319,7 +26319,7 @@
       </c>
       <c r="V336" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12031.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12031.png</t>
         </is>
       </c>
     </row>
@@ -26396,7 +26396,7 @@
       </c>
       <c r="V337" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12080.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12080.jpg</t>
         </is>
       </c>
     </row>
@@ -26473,7 +26473,7 @@
       </c>
       <c r="V338" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12098.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12098.jpg</t>
         </is>
       </c>
     </row>
@@ -26627,7 +26627,7 @@
       </c>
       <c r="V340" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12105.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12105.jpg</t>
         </is>
       </c>
     </row>
@@ -26704,7 +26704,7 @@
       </c>
       <c r="V341" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12106.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12106.jpg</t>
         </is>
       </c>
     </row>
@@ -26781,7 +26781,7 @@
       </c>
       <c r="V342" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12107.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12107.jpg</t>
         </is>
       </c>
     </row>
@@ -26858,7 +26858,7 @@
       </c>
       <c r="V343" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12108.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12108.jpg</t>
         </is>
       </c>
     </row>
@@ -27012,7 +27012,7 @@
       </c>
       <c r="V345" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12096.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12096.png</t>
         </is>
       </c>
     </row>
@@ -27166,7 +27166,7 @@
       </c>
       <c r="V347" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12119.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12119.jpg</t>
         </is>
       </c>
     </row>
@@ -27320,7 +27320,7 @@
       </c>
       <c r="V349" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12145.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12145.webp</t>
         </is>
       </c>
     </row>
@@ -27551,7 +27551,7 @@
       </c>
       <c r="V352" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12148.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12148.jpg</t>
         </is>
       </c>
     </row>
@@ -27628,7 +27628,7 @@
       </c>
       <c r="V353" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12160.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12160.jpg</t>
         </is>
       </c>
     </row>
@@ -27705,7 +27705,7 @@
       </c>
       <c r="V354" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12161.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12161.jpg</t>
         </is>
       </c>
     </row>
@@ -27782,7 +27782,7 @@
       </c>
       <c r="V355" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12162.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12162.png</t>
         </is>
       </c>
     </row>
@@ -27859,7 +27859,7 @@
       </c>
       <c r="V356" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12164.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12164.png</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
UND empacotado + granel solto
</commit_message>
<xml_diff>
--- a/PLANILHA-FOTOS-NOVAS-355.xlsx
+++ b/PLANILHA-FOTOS-NOVAS-355.xlsx
@@ -755,7 +755,7 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/adocantes-naturais/11817.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/adocantes-naturais/11817.jpg</t>
         </is>
       </c>
     </row>
@@ -909,7 +909,7 @@
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/adocantes-naturais/12027.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/adocantes-naturais/12027.webp</t>
         </is>
       </c>
     </row>
@@ -986,7 +986,7 @@
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/adocantes-naturais/12028.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/adocantes-naturais/12028.jpg</t>
         </is>
       </c>
     </row>
@@ -1448,7 +1448,7 @@
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10255.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10255.webp</t>
         </is>
       </c>
     </row>
@@ -1910,7 +1910,7 @@
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10866.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10866.jpg</t>
         </is>
       </c>
     </row>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10900.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10900.webp</t>
         </is>
       </c>
     </row>
@@ -2141,7 +2141,7 @@
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10901.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10901.webp</t>
         </is>
       </c>
     </row>
@@ -2526,7 +2526,7 @@
       </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10957.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10957.png</t>
         </is>
       </c>
     </row>
@@ -2603,7 +2603,7 @@
       </c>
       <c r="V28" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10978.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10978.jpg</t>
         </is>
       </c>
     </row>
@@ -2680,7 +2680,7 @@
       </c>
       <c r="V29" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11005.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11005.webp</t>
         </is>
       </c>
     </row>
@@ -2757,7 +2757,7 @@
       </c>
       <c r="V30" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11054.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11054.png</t>
         </is>
       </c>
     </row>
@@ -2834,7 +2834,7 @@
       </c>
       <c r="V31" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11055.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11055.webp</t>
         </is>
       </c>
     </row>
@@ -3219,7 +3219,7 @@
       </c>
       <c r="V36" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11091.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11091.jpg</t>
         </is>
       </c>
     </row>
@@ -3296,7 +3296,7 @@
       </c>
       <c r="V37" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11092.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11092.jpg</t>
         </is>
       </c>
     </row>
@@ -3527,7 +3527,7 @@
       </c>
       <c r="V40" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11120.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11120.jpg</t>
         </is>
       </c>
     </row>
@@ -3604,7 +3604,7 @@
       </c>
       <c r="V41" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11121.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11121.jpg</t>
         </is>
       </c>
     </row>
@@ -3681,7 +3681,7 @@
       </c>
       <c r="V42" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11124.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11124.webp</t>
         </is>
       </c>
     </row>
@@ -3912,7 +3912,7 @@
       </c>
       <c r="V45" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11136.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11136.jpg</t>
         </is>
       </c>
     </row>
@@ -4451,7 +4451,7 @@
       </c>
       <c r="V52" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11326.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11326.jpg</t>
         </is>
       </c>
     </row>
@@ -4528,7 +4528,7 @@
       </c>
       <c r="V53" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11329.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11329.png</t>
         </is>
       </c>
     </row>
@@ -4759,7 +4759,7 @@
       </c>
       <c r="V56" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11334.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11334.jpg</t>
         </is>
       </c>
     </row>
@@ -4913,7 +4913,7 @@
       </c>
       <c r="V58" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11337.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11337.jpg</t>
         </is>
       </c>
     </row>
@@ -4990,7 +4990,7 @@
       </c>
       <c r="V59" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11338.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11338.jpg</t>
         </is>
       </c>
     </row>
@@ -5067,7 +5067,7 @@
       </c>
       <c r="V60" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11339.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11339.png</t>
         </is>
       </c>
     </row>
@@ -5375,7 +5375,7 @@
       </c>
       <c r="V64" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11400.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11400.webp</t>
         </is>
       </c>
     </row>
@@ -5529,7 +5529,7 @@
       </c>
       <c r="V66" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11402.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11402.webp</t>
         </is>
       </c>
     </row>
@@ -5760,7 +5760,7 @@
       </c>
       <c r="V69" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/12091.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/12091.webp</t>
         </is>
       </c>
     </row>
@@ -5914,7 +5914,7 @@
       </c>
       <c r="V71" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/12158.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/12158.jpg</t>
         </is>
       </c>
     </row>
@@ -5991,7 +5991,7 @@
       </c>
       <c r="V72" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/12175.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/12175.jpg</t>
         </is>
       </c>
     </row>
@@ -6145,7 +6145,7 @@
       </c>
       <c r="V74" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/10037.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/10037.webp</t>
         </is>
       </c>
     </row>
@@ -6222,7 +6222,7 @@
       </c>
       <c r="V75" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/10044.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/10044.jpg</t>
         </is>
       </c>
     </row>
@@ -6376,7 +6376,7 @@
       </c>
       <c r="V77" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/10073.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/10073.jpg</t>
         </is>
       </c>
     </row>
@@ -6684,7 +6684,7 @@
       </c>
       <c r="V81" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11848.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11848.jpg</t>
         </is>
       </c>
     </row>
@@ -6838,7 +6838,7 @@
       </c>
       <c r="V83" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11902.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11902.jpg</t>
         </is>
       </c>
     </row>
@@ -6915,7 +6915,7 @@
       </c>
       <c r="V84" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11939.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11939.webp</t>
         </is>
       </c>
     </row>
@@ -6992,7 +6992,7 @@
       </c>
       <c r="V85" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11996.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11996.jpg</t>
         </is>
       </c>
     </row>
@@ -7069,7 +7069,7 @@
       </c>
       <c r="V86" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11998.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11998.png</t>
         </is>
       </c>
     </row>
@@ -7223,7 +7223,7 @@
       </c>
       <c r="V88" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/12071.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/12071.jpg</t>
         </is>
       </c>
     </row>
@@ -7531,7 +7531,7 @@
       </c>
       <c r="V92" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/10278.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/10278.jpg</t>
         </is>
       </c>
     </row>
@@ -7608,7 +7608,7 @@
       </c>
       <c r="V93" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/10873.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/10873.png</t>
         </is>
       </c>
     </row>
@@ -7839,7 +7839,7 @@
       </c>
       <c r="V96" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/11898.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/11898.jpg</t>
         </is>
       </c>
     </row>
@@ -7916,7 +7916,7 @@
       </c>
       <c r="V97" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/11940.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/11940.jpg</t>
         </is>
       </c>
     </row>
@@ -7993,7 +7993,7 @@
       </c>
       <c r="V98" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/11941.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/11941.jpg</t>
         </is>
       </c>
     </row>
@@ -8070,7 +8070,7 @@
       </c>
       <c r="V99" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/11951.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/11951.png</t>
         </is>
       </c>
     </row>
@@ -8917,7 +8917,7 @@
       </c>
       <c r="V110" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11809.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11809.png</t>
         </is>
       </c>
     </row>
@@ -9225,7 +9225,7 @@
       </c>
       <c r="V114" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11868.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11868.png</t>
         </is>
       </c>
     </row>
@@ -10303,7 +10303,7 @@
       </c>
       <c r="V128" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11490.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11490.png</t>
         </is>
       </c>
     </row>
@@ -12151,7 +12151,7 @@
       </c>
       <c r="V152" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11778.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11778.png</t>
         </is>
       </c>
     </row>
@@ -13306,7 +13306,7 @@
       </c>
       <c r="V167" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11796.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11796.jpg</t>
         </is>
       </c>
     </row>
@@ -15693,7 +15693,7 @@
       </c>
       <c r="V198" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/12053.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/12053.webp</t>
         </is>
       </c>
     </row>
@@ -15847,7 +15847,7 @@
       </c>
       <c r="V200" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/12151.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/12151.png</t>
         </is>
       </c>
     </row>
@@ -16309,7 +16309,7 @@
       </c>
       <c r="V206" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11536.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11536.webp</t>
         </is>
       </c>
     </row>
@@ -17079,7 +17079,7 @@
       </c>
       <c r="V216" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11735.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11735.png</t>
         </is>
       </c>
     </row>
@@ -17310,7 +17310,7 @@
       </c>
       <c r="V219" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11741.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11741.webp</t>
         </is>
       </c>
     </row>
@@ -18003,7 +18003,7 @@
       </c>
       <c r="V228" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11804.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11804.jpg</t>
         </is>
       </c>
     </row>
@@ -18388,7 +18388,7 @@
       </c>
       <c r="V233" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11959.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11959.jpg</t>
         </is>
       </c>
     </row>
@@ -19928,7 +19928,7 @@
       </c>
       <c r="V253" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/11865.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/11865.webp</t>
         </is>
       </c>
     </row>
@@ -20775,7 +20775,7 @@
       </c>
       <c r="V264" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10887.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10887.jpg</t>
         </is>
       </c>
     </row>
@@ -20852,7 +20852,7 @@
       </c>
       <c r="V265" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10902.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10902.jpg</t>
         </is>
       </c>
     </row>
@@ -22007,7 +22007,7 @@
       </c>
       <c r="V280" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11499.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11499.jpg</t>
         </is>
       </c>
     </row>
@@ -23393,7 +23393,7 @@
       </c>
       <c r="V298" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11607.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11607.png</t>
         </is>
       </c>
     </row>
@@ -25549,7 +25549,7 @@
       </c>
       <c r="V326" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11910.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11910.webp</t>
         </is>
       </c>
     </row>
@@ -25626,7 +25626,7 @@
       </c>
       <c r="V327" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11913.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11913.webp</t>
         </is>
       </c>
     </row>
@@ -26011,7 +26011,7 @@
       </c>
       <c r="V332" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12010.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12010.jpg</t>
         </is>
       </c>
     </row>
@@ -26319,7 +26319,7 @@
       </c>
       <c r="V336" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12031.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12031.jpg</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
classificacao por nome: qtd/marca=pacote, resto granel
</commit_message>
<xml_diff>
--- a/PLANILHA-FOTOS-NOVAS-355.xlsx
+++ b/PLANILHA-FOTOS-NOVAS-355.xlsx
@@ -986,7 +986,7 @@
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/adocantes-naturais/12028.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/adocantes-naturais/12028.webp</t>
         </is>
       </c>
     </row>
@@ -1833,7 +1833,7 @@
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10745.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10745.png</t>
         </is>
       </c>
     </row>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10900.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10900.jpg</t>
         </is>
       </c>
     </row>
@@ -2141,7 +2141,7 @@
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10901.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10901.jpg</t>
         </is>
       </c>
     </row>
@@ -2526,7 +2526,7 @@
       </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10957.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/10957.jpg</t>
         </is>
       </c>
     </row>
@@ -2834,7 +2834,7 @@
       </c>
       <c r="V31" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11055.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11055.jpg</t>
         </is>
       </c>
     </row>
@@ -3527,7 +3527,7 @@
       </c>
       <c r="V40" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11120.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11120.webp</t>
         </is>
       </c>
     </row>
@@ -3681,7 +3681,7 @@
       </c>
       <c r="V42" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11124.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11124.jpg</t>
         </is>
       </c>
     </row>
@@ -3912,7 +3912,7 @@
       </c>
       <c r="V45" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11136.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11136.png</t>
         </is>
       </c>
     </row>
@@ -5067,7 +5067,7 @@
       </c>
       <c r="V60" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11339.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/11339.jpg</t>
         </is>
       </c>
     </row>
@@ -5914,7 +5914,7 @@
       </c>
       <c r="V71" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/12158.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/12158.webp</t>
         </is>
       </c>
     </row>
@@ -6145,7 +6145,7 @@
       </c>
       <c r="V74" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/10037.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/10037.jpg</t>
         </is>
       </c>
     </row>
@@ -6222,7 +6222,7 @@
       </c>
       <c r="V75" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/10044.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/10044.png</t>
         </is>
       </c>
     </row>
@@ -6838,7 +6838,7 @@
       </c>
       <c r="V83" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11902.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11902.png</t>
         </is>
       </c>
     </row>
@@ -6915,7 +6915,7 @@
       </c>
       <c r="V84" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11939.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11939.jpg</t>
         </is>
       </c>
     </row>
@@ -6992,7 +6992,7 @@
       </c>
       <c r="V85" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11996.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11996.webp</t>
         </is>
       </c>
     </row>
@@ -7069,7 +7069,7 @@
       </c>
       <c r="V86" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11998.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11998.jpg</t>
         </is>
       </c>
     </row>
@@ -7223,7 +7223,7 @@
       </c>
       <c r="V88" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/12071.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/12071.webp</t>
         </is>
       </c>
     </row>
@@ -7608,7 +7608,7 @@
       </c>
       <c r="V93" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/10873.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/10873.jpg</t>
         </is>
       </c>
     </row>
@@ -7685,7 +7685,7 @@
       </c>
       <c r="V94" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/11480.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/11480.webp</t>
         </is>
       </c>
     </row>
@@ -7839,7 +7839,7 @@
       </c>
       <c r="V96" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/11898.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/11898.png</t>
         </is>
       </c>
     </row>
@@ -7993,7 +7993,7 @@
       </c>
       <c r="V98" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/11941.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/11941.webp</t>
         </is>
       </c>
     </row>
@@ -10457,7 +10457,7 @@
       </c>
       <c r="V130" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11553.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11553.jpg</t>
         </is>
       </c>
     </row>
@@ -10996,7 +10996,7 @@
       </c>
       <c r="V137" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11753.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11753.png</t>
         </is>
       </c>
     </row>
@@ -12767,7 +12767,7 @@
       </c>
       <c r="V160" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11787.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11787.png</t>
         </is>
       </c>
     </row>
@@ -12998,7 +12998,7 @@
       </c>
       <c r="V163" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11791.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11791.jpg</t>
         </is>
       </c>
     </row>
@@ -13537,7 +13537,7 @@
       </c>
       <c r="V170" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11966.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11966.png</t>
         </is>
       </c>
     </row>
@@ -14076,7 +14076,7 @@
       </c>
       <c r="V177" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11446.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11446.webp</t>
         </is>
       </c>
     </row>
@@ -14153,7 +14153,7 @@
       </c>
       <c r="V178" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11447.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11447.webp</t>
         </is>
       </c>
     </row>
@@ -16232,7 +16232,7 @@
       </c>
       <c r="V205" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11535.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11535.webp</t>
         </is>
       </c>
     </row>
@@ -17079,7 +17079,7 @@
       </c>
       <c r="V216" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11735.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11735.jpg</t>
         </is>
       </c>
     </row>
@@ -17695,7 +17695,7 @@
       </c>
       <c r="V224" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11748.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11748.jpg</t>
         </is>
       </c>
     </row>
@@ -18003,7 +18003,7 @@
       </c>
       <c r="V228" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11804.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11804.webp</t>
         </is>
       </c>
     </row>
@@ -18234,7 +18234,7 @@
       </c>
       <c r="V231" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11957.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11957.webp</t>
         </is>
       </c>
     </row>
@@ -18388,7 +18388,7 @@
       </c>
       <c r="V233" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11959.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11959.webp</t>
         </is>
       </c>
     </row>
@@ -18619,7 +18619,7 @@
       </c>
       <c r="V236" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11962.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/11962.webp</t>
         </is>
       </c>
     </row>
@@ -18927,7 +18927,7 @@
       </c>
       <c r="V240" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/12101.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/graos/12101.webp</t>
         </is>
       </c>
     </row>
@@ -19235,7 +19235,7 @@
       </c>
       <c r="V244" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/11184.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/sementes/11184.webp</t>
         </is>
       </c>
     </row>
@@ -20082,7 +20082,7 @@
       </c>
       <c r="V255" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10061.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10061.webp</t>
         </is>
       </c>
     </row>
@@ -20313,7 +20313,7 @@
       </c>
       <c r="V258" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10256.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10256.jpg</t>
         </is>
       </c>
     </row>
@@ -20467,7 +20467,7 @@
       </c>
       <c r="V260" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10306.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10306.webp</t>
         </is>
       </c>
     </row>
@@ -20852,7 +20852,7 @@
       </c>
       <c r="V265" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10902.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10902.png</t>
         </is>
       </c>
     </row>
@@ -21391,7 +21391,7 @@
       </c>
       <c r="V272" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11382.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11382.jpg</t>
         </is>
       </c>
     </row>
@@ -22315,7 +22315,7 @@
       </c>
       <c r="V284" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11563.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11563.jpg</t>
         </is>
       </c>
     </row>
@@ -25549,7 +25549,7 @@
       </c>
       <c r="V326" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11910.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11910.png</t>
         </is>
       </c>
     </row>
@@ -27705,7 +27705,7 @@
       </c>
       <c r="V354" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12161.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12161.webp</t>
         </is>
       </c>
     </row>
@@ -27859,7 +27859,7 @@
       </c>
       <c r="V356" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12164.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12164.jpg</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
verificacao 1-a-1: 73 trocas + xylitol
</commit_message>
<xml_diff>
--- a/PLANILHA-FOTOS-NOVAS-355.xlsx
+++ b/PLANILHA-FOTOS-NOVAS-355.xlsx
@@ -12151,7 +12151,7 @@
       </c>
       <c r="V152" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11779.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11779.webp</t>
         </is>
       </c>
     </row>
@@ -12536,7 +12536,7 @@
       </c>
       <c r="V157" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11784.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11784.jpg</t>
         </is>
       </c>
     </row>
@@ -13383,7 +13383,7 @@
       </c>
       <c r="V168" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11953.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11953.png</t>
         </is>
       </c>
     </row>
@@ -20005,7 +20005,7 @@
       </c>
       <c r="V254" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10061.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10061.jpg</t>
         </is>
       </c>
     </row>
@@ -20159,7 +20159,7 @@
       </c>
       <c r="V256" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10171.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10171.jpg</t>
         </is>
       </c>
     </row>
@@ -21314,7 +21314,7 @@
       </c>
       <c r="V271" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11382.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11382.jpg</t>
         </is>
       </c>
     </row>
@@ -21622,7 +21622,7 @@
       </c>
       <c r="V275" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11487.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11487.jpg</t>
         </is>
       </c>
     </row>
@@ -22623,7 +22623,7 @@
       </c>
       <c r="V288" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11570.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11570.jpg</t>
         </is>
       </c>
     </row>
@@ -23778,7 +23778,7 @@
       </c>
       <c r="V303" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11647.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11647.jpg</t>
         </is>
       </c>
     </row>
@@ -25626,7 +25626,7 @@
       </c>
       <c r="V327" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11931.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11931.webp</t>
         </is>
       </c>
     </row>
@@ -26858,7 +26858,7 @@
       </c>
       <c r="V343" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12096.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12096.jpg</t>
         </is>
       </c>
     </row>
@@ -27089,7 +27089,7 @@
       </c>
       <c r="V346" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12115.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12115.jpg</t>
         </is>
       </c>
     </row>
@@ -27320,7 +27320,7 @@
       </c>
       <c r="V349" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12147.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12147.jpg</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
2 finais ok - todas corretas
</commit_message>
<xml_diff>
--- a/PLANILHA-FOTOS-NOVAS-355.xlsx
+++ b/PLANILHA-FOTOS-NOVAS-355.xlsx
@@ -20005,7 +20005,7 @@
       </c>
       <c r="V254" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10061.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10061.png</t>
         </is>
       </c>
     </row>
@@ -27089,7 +27089,7 @@
       </c>
       <c r="V346" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12115.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12115.png</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
revisao 1a1 completa: banco limpo
</commit_message>
<xml_diff>
--- a/PLANILHA-FOTOS-NOVAS-355.xlsx
+++ b/PLANILHA-FOTOS-NOVAS-355.xlsx
@@ -1063,7 +1063,7 @@
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/adocantes-naturais/12174.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/adocantes-naturais/12174.jpg</t>
         </is>
       </c>
     </row>
@@ -6992,7 +6992,7 @@
       </c>
       <c r="V85" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11996.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11996.jpg</t>
         </is>
       </c>
     </row>
@@ -7069,7 +7069,7 @@
       </c>
       <c r="V86" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11998.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/chips-e-snacks/11998.jpg</t>
         </is>
       </c>
     </row>
@@ -8224,7 +8224,7 @@
       </c>
       <c r="V101" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/10944.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/10944.jpg</t>
         </is>
       </c>
     </row>
@@ -8455,7 +8455,7 @@
       </c>
       <c r="V104" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11594.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11594.png</t>
         </is>
       </c>
     </row>
@@ -9225,7 +9225,7 @@
       </c>
       <c r="V114" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11868.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11868.jpg</t>
         </is>
       </c>
     </row>
@@ -9764,7 +9764,7 @@
       </c>
       <c r="V121" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11968.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/11968.png</t>
         </is>
       </c>
     </row>
@@ -11689,7 +11689,7 @@
       </c>
       <c r="V146" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11771.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11771.jpg</t>
         </is>
       </c>
     </row>
@@ -11843,7 +11843,7 @@
       </c>
       <c r="V148" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11774.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11774.jpg</t>
         </is>
       </c>
     </row>
@@ -12151,7 +12151,7 @@
       </c>
       <c r="V152" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11779.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11779.jpg</t>
         </is>
       </c>
     </row>
@@ -12767,7 +12767,7 @@
       </c>
       <c r="V160" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11789.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11789.png</t>
         </is>
       </c>
     </row>
@@ -13537,7 +13537,7 @@
       </c>
       <c r="V170" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11972.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11972.jpg</t>
         </is>
       </c>
     </row>
@@ -22469,7 +22469,7 @@
       </c>
       <c r="V286" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11568.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11568.jpg</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
drageados + especificos + codigos certos
</commit_message>
<xml_diff>
--- a/PLANILHA-FOTOS-NOVAS-355.xlsx
+++ b/PLANILHA-FOTOS-NOVAS-355.xlsx
@@ -7685,7 +7685,7 @@
       </c>
       <c r="V94" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/11480.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/11480.png</t>
         </is>
       </c>
     </row>
@@ -7839,7 +7839,7 @@
       </c>
       <c r="V96" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/11898.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/11898.jpg</t>
         </is>
       </c>
     </row>
@@ -7916,7 +7916,7 @@
       </c>
       <c r="V97" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/11940.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/drageados/11940.webp</t>
         </is>
       </c>
     </row>
@@ -8147,7 +8147,7 @@
       </c>
       <c r="V100" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/10886.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/ervas/10886.webp</t>
         </is>
       </c>
     </row>
@@ -11304,7 +11304,7 @@
       </c>
       <c r="V141" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11762.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11762.jpg</t>
         </is>
       </c>
     </row>
@@ -11458,7 +11458,7 @@
       </c>
       <c r="V143" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11765.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11765.jpg</t>
         </is>
       </c>
     </row>
@@ -11535,7 +11535,7 @@
       </c>
       <c r="V144" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11767.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11767.jpg</t>
         </is>
       </c>
     </row>
@@ -12074,7 +12074,7 @@
       </c>
       <c r="V151" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11778.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11778.jpg</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
multi-opcao nos 6 teimosos
</commit_message>
<xml_diff>
--- a/PLANILHA-FOTOS-NOVAS-355.xlsx
+++ b/PLANILHA-FOTOS-NOVAS-355.xlsx
@@ -6068,7 +6068,7 @@
       </c>
       <c r="V73" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/12176.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/apicultura/12176.jpg</t>
         </is>
       </c>
     </row>
@@ -23778,7 +23778,7 @@
       </c>
       <c r="V303" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11655.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11655.jpg</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
5 trocas marca + coentro desidratado + 2 desativados
</commit_message>
<xml_diff>
--- a/PLANILHA-FOTOS-NOVAS-355.xlsx
+++ b/PLANILHA-FOTOS-NOVAS-355.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF351"/>
+  <dimension ref="A1:AF349"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11304,7 +11304,7 @@
       </c>
       <c r="V141" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11763.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11763.jpg</t>
         </is>
       </c>
     </row>
@@ -19934,21 +19934,21 @@
     </row>
     <row r="254">
       <c r="A254" t="n">
-        <v>10171</v>
+        <v>10256</v>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>10171</t>
+          <t>10256</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>LEMON C/ ERVAS FINAS 500G</t>
+          <t>OREGANO EM PO 20G</t>
         </is>
       </c>
       <c r="F254" t="inlineStr">
         <is>
-          <t>UNI</t>
+          <t>KG</t>
         </is>
       </c>
       <c r="G254" t="n">
@@ -19958,10 +19958,10 @@
         <v>10</v>
       </c>
       <c r="I254" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="J254" t="n">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="K254" t="inlineStr">
         <is>
@@ -19979,10 +19979,10 @@
         </is>
       </c>
       <c r="N254" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="O254" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="P254" t="n">
         <v>0</v>
@@ -19996,31 +19996,31 @@
         </is>
       </c>
       <c r="T254" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="U254" t="inlineStr">
         <is>
-          <t>UND</t>
+          <t>100g</t>
         </is>
       </c>
       <c r="V254" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10171.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10256.webp</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="n">
-        <v>10256</v>
+        <v>10264</v>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>10256</t>
+          <t>2145</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>OREGANO EM PO 20G</t>
+          <t>MANJERICAO EM PO</t>
         </is>
       </c>
       <c r="F255" t="inlineStr">
@@ -20056,10 +20056,10 @@
         </is>
       </c>
       <c r="N255" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="O255" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="P255" t="n">
         <v>0</v>
@@ -20082,22 +20082,22 @@
       </c>
       <c r="V255" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10256.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10264.jpg</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="n">
-        <v>10264</v>
+        <v>10306</v>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2145</t>
+          <t>2121</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>MANJERICAO EM PO</t>
+          <t>CANELA PO PURA PREMIUM</t>
         </is>
       </c>
       <c r="F256" t="inlineStr">
@@ -20133,10 +20133,10 @@
         </is>
       </c>
       <c r="N256" t="n">
-        <v>20</v>
+        <v>105</v>
       </c>
       <c r="O256" t="n">
-        <v>20</v>
+        <v>105</v>
       </c>
       <c r="P256" t="n">
         <v>0</v>
@@ -20159,22 +20159,22 @@
       </c>
       <c r="V256" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10264.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10306.jpg</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="n">
-        <v>10306</v>
+        <v>10308</v>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2121</t>
+          <t>1333</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>CANELA PO PURA PREMIUM</t>
+          <t>CHIMICHURRI DEFUMADO</t>
         </is>
       </c>
       <c r="F257" t="inlineStr">
@@ -20210,10 +20210,10 @@
         </is>
       </c>
       <c r="N257" t="n">
-        <v>105</v>
+        <v>65</v>
       </c>
       <c r="O257" t="n">
-        <v>105</v>
+        <v>65</v>
       </c>
       <c r="P257" t="n">
         <v>0</v>
@@ -20236,22 +20236,22 @@
       </c>
       <c r="V257" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10306.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10308.jpg</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="n">
-        <v>10308</v>
+        <v>10550</v>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>1333</t>
+          <t>2305</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>CHIMICHURRI DEFUMADO</t>
+          <t>ORANGE PEPPER</t>
         </is>
       </c>
       <c r="F258" t="inlineStr">
@@ -20287,10 +20287,10 @@
         </is>
       </c>
       <c r="N258" t="n">
-        <v>65</v>
+        <v>48</v>
       </c>
       <c r="O258" t="n">
-        <v>65</v>
+        <v>48</v>
       </c>
       <c r="P258" t="n">
         <v>0</v>
@@ -20313,22 +20313,22 @@
       </c>
       <c r="V258" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10308.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10550.png</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="n">
-        <v>10550</v>
+        <v>10720</v>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2305</t>
+          <t>338</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>ORANGE PEPPER</t>
+          <t>ALHO ROXO SOLTO</t>
         </is>
       </c>
       <c r="F259" t="inlineStr">
@@ -20364,10 +20364,10 @@
         </is>
       </c>
       <c r="N259" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="O259" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="P259" t="n">
         <v>0</v>
@@ -20390,22 +20390,22 @@
       </c>
       <c r="V259" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10550.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10720.jpg</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="n">
-        <v>10720</v>
+        <v>10887</v>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>338</t>
+          <t>308</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>ALHO ROXO SOLTO</t>
+          <t>ACAFRAO IMPORTADO</t>
         </is>
       </c>
       <c r="F260" t="inlineStr">
@@ -20441,10 +20441,10 @@
         </is>
       </c>
       <c r="N260" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="O260" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="P260" t="n">
         <v>0</v>
@@ -20467,22 +20467,22 @@
       </c>
       <c r="V260" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10720.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10887.jpg</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="n">
-        <v>10887</v>
+        <v>10902</v>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>308</t>
+          <t>173</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>ACAFRAO IMPORTADO</t>
+          <t>TEMPERO BAIANO SEM PIMENTA</t>
         </is>
       </c>
       <c r="F261" t="inlineStr">
@@ -20518,10 +20518,10 @@
         </is>
       </c>
       <c r="N261" t="n">
-        <v>50</v>
+        <v>11.5</v>
       </c>
       <c r="O261" t="n">
-        <v>50</v>
+        <v>11.5</v>
       </c>
       <c r="P261" t="n">
         <v>0</v>
@@ -20544,22 +20544,22 @@
       </c>
       <c r="V261" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10887.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10902.jpg</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="n">
-        <v>10902</v>
+        <v>10967</v>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>173</t>
+          <t>305</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>TEMPERO BAIANO SEM PIMENTA</t>
+          <t>CREME DE CEBOLA</t>
         </is>
       </c>
       <c r="F262" t="inlineStr">
@@ -20595,10 +20595,10 @@
         </is>
       </c>
       <c r="N262" t="n">
-        <v>11.5</v>
+        <v>20</v>
       </c>
       <c r="O262" t="n">
-        <v>11.5</v>
+        <v>20</v>
       </c>
       <c r="P262" t="n">
         <v>0</v>
@@ -20621,22 +20621,22 @@
       </c>
       <c r="V262" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10902.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10967.jpg</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="n">
-        <v>10967</v>
+        <v>11029</v>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>305</t>
+          <t>352</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>CREME DE CEBOLA</t>
+          <t>CEBOLA CRISPY</t>
         </is>
       </c>
       <c r="F263" t="inlineStr">
@@ -20672,10 +20672,10 @@
         </is>
       </c>
       <c r="N263" t="n">
-        <v>20</v>
+        <v>125</v>
       </c>
       <c r="O263" t="n">
-        <v>20</v>
+        <v>125</v>
       </c>
       <c r="P263" t="n">
         <v>0</v>
@@ -20698,22 +20698,22 @@
       </c>
       <c r="V263" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/10967.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11029.webp</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="n">
-        <v>11029</v>
+        <v>11167</v>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>352</t>
+          <t>6033</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>CEBOLA CRISPY</t>
+          <t>FIT EDU GUEDES</t>
         </is>
       </c>
       <c r="F264" t="inlineStr">
@@ -20749,10 +20749,10 @@
         </is>
       </c>
       <c r="N264" t="n">
-        <v>125</v>
+        <v>48</v>
       </c>
       <c r="O264" t="n">
-        <v>125</v>
+        <v>48</v>
       </c>
       <c r="P264" t="n">
         <v>0</v>
@@ -20775,22 +20775,22 @@
       </c>
       <c r="V264" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11029.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11167.jpg</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="n">
-        <v>11167</v>
+        <v>11168</v>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>6033</t>
+          <t>6031</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>FIT EDU GUEDES</t>
+          <t>TEMPERO MINEIRO</t>
         </is>
       </c>
       <c r="F265" t="inlineStr">
@@ -20826,10 +20826,10 @@
         </is>
       </c>
       <c r="N265" t="n">
-        <v>48</v>
+        <v>25</v>
       </c>
       <c r="O265" t="n">
-        <v>48</v>
+        <v>25</v>
       </c>
       <c r="P265" t="n">
         <v>0</v>
@@ -20852,22 +20852,22 @@
       </c>
       <c r="V265" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11167.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11168.jpg</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="n">
-        <v>11168</v>
+        <v>11170</v>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>6031</t>
+          <t>6029</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>TEMPERO MINEIRO</t>
+          <t>FIT COMPLETO</t>
         </is>
       </c>
       <c r="F266" t="inlineStr">
@@ -20903,10 +20903,10 @@
         </is>
       </c>
       <c r="N266" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="O266" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="P266" t="n">
         <v>0</v>
@@ -20929,22 +20929,22 @@
       </c>
       <c r="V266" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11168.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11170.jpg</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="n">
-        <v>11170</v>
+        <v>11237</v>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>6029</t>
+          <t>4415</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>FIT COMPLETO</t>
+          <t>TEMPERO SIRIO</t>
         </is>
       </c>
       <c r="F267" t="inlineStr">
@@ -20980,10 +20980,10 @@
         </is>
       </c>
       <c r="N267" t="n">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="O267" t="n">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="P267" t="n">
         <v>0</v>
@@ -21006,22 +21006,22 @@
       </c>
       <c r="V267" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11170.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11237.jpg</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="n">
-        <v>11237</v>
+        <v>11466</v>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>4415</t>
+          <t>3797</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>TEMPERO SIRIO</t>
+          <t>ZIMBRO</t>
         </is>
       </c>
       <c r="F268" t="inlineStr">
@@ -21057,10 +21057,10 @@
         </is>
       </c>
       <c r="N268" t="n">
-        <v>38</v>
+        <v>229</v>
       </c>
       <c r="O268" t="n">
-        <v>38</v>
+        <v>229</v>
       </c>
       <c r="P268" t="n">
         <v>0</v>
@@ -21083,40 +21083,40 @@
       </c>
       <c r="V268" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11237.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11466.jpg</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="n">
-        <v>11382</v>
+        <v>11468</v>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>4019</t>
+          <t>971</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>GARAM MASALA 20G</t>
+          <t>ZATTAR</t>
         </is>
       </c>
       <c r="F269" t="inlineStr">
         <is>
-          <t>UN</t>
+          <t>KG</t>
         </is>
       </c>
       <c r="G269" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="H269" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="I269" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="J269" t="n">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="K269" t="inlineStr">
         <is>
@@ -21134,10 +21134,10 @@
         </is>
       </c>
       <c r="N269" t="n">
-        <v>2.5</v>
+        <v>55</v>
       </c>
       <c r="O269" t="n">
-        <v>2.5</v>
+        <v>55</v>
       </c>
       <c r="P269" t="n">
         <v>0</v>
@@ -21151,31 +21151,31 @@
         </is>
       </c>
       <c r="T269" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="U269" t="inlineStr">
         <is>
-          <t>UND</t>
+          <t>100g</t>
         </is>
       </c>
       <c r="V269" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11382.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11468.webp</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="n">
-        <v>11466</v>
+        <v>11473</v>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>3797</t>
+          <t>91</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>ZIMBRO</t>
+          <t>VINAGRETE</t>
         </is>
       </c>
       <c r="F270" t="inlineStr">
@@ -21211,10 +21211,10 @@
         </is>
       </c>
       <c r="N270" t="n">
-        <v>229</v>
+        <v>68</v>
       </c>
       <c r="O270" t="n">
-        <v>229</v>
+        <v>68</v>
       </c>
       <c r="P270" t="n">
         <v>0</v>
@@ -21237,22 +21237,22 @@
       </c>
       <c r="V270" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11466.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11473.jpg</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="n">
-        <v>11468</v>
+        <v>11487</v>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>971</t>
+          <t>1522</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>ZATTAR</t>
+          <t>PEGA MARIDO</t>
         </is>
       </c>
       <c r="F271" t="inlineStr">
@@ -21288,10 +21288,10 @@
         </is>
       </c>
       <c r="N271" t="n">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="O271" t="n">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="P271" t="n">
         <v>0</v>
@@ -21314,22 +21314,22 @@
       </c>
       <c r="V271" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11468.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11487.jpg</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="n">
-        <v>11473</v>
+        <v>11493</v>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>3437</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>VINAGRETE</t>
+          <t>TOMILHO</t>
         </is>
       </c>
       <c r="F272" t="inlineStr">
@@ -21365,10 +21365,10 @@
         </is>
       </c>
       <c r="N272" t="n">
-        <v>68</v>
+        <v>29</v>
       </c>
       <c r="O272" t="n">
-        <v>68</v>
+        <v>29</v>
       </c>
       <c r="P272" t="n">
         <v>0</v>
@@ -21391,22 +21391,22 @@
       </c>
       <c r="V272" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11473.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11493.jpg</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="n">
-        <v>11487</v>
+        <v>11496</v>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>1522</t>
+          <t>92</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>PEGA MARIDO</t>
+          <t>TEMPERO FEIJAO</t>
         </is>
       </c>
       <c r="F273" t="inlineStr">
@@ -21442,10 +21442,10 @@
         </is>
       </c>
       <c r="N273" t="n">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="O273" t="n">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="P273" t="n">
         <v>0</v>
@@ -21468,22 +21468,22 @@
       </c>
       <c r="V273" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11487.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11496.jpg</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="n">
-        <v>11493</v>
+        <v>11497</v>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>3437</t>
+          <t>3593</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>TOMILHO</t>
+          <t>LEMON COM ERVAS FINAS</t>
         </is>
       </c>
       <c r="F274" t="inlineStr">
@@ -21519,10 +21519,10 @@
         </is>
       </c>
       <c r="N274" t="n">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="O274" t="n">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="P274" t="n">
         <v>0</v>
@@ -21545,22 +21545,22 @@
       </c>
       <c r="V274" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11493.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11497.png</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="n">
-        <v>11496</v>
+        <v>11499</v>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>92</t>
+          <t>78</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>TEMPERO FEIJAO</t>
+          <t>TEMPERO BAIANO PO</t>
         </is>
       </c>
       <c r="F275" t="inlineStr">
@@ -21596,10 +21596,10 @@
         </is>
       </c>
       <c r="N275" t="n">
-        <v>50</v>
+        <v>13</v>
       </c>
       <c r="O275" t="n">
-        <v>50</v>
+        <v>13</v>
       </c>
       <c r="P275" t="n">
         <v>0</v>
@@ -21622,22 +21622,22 @@
       </c>
       <c r="V275" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11496.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11499.jpg</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="n">
-        <v>11497</v>
+        <v>11500</v>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>3593</t>
+          <t>79</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>LEMON COM ERVAS FINAS</t>
+          <t>TEMPERO BAIANO GRAO</t>
         </is>
       </c>
       <c r="F276" t="inlineStr">
@@ -21673,10 +21673,10 @@
         </is>
       </c>
       <c r="N276" t="n">
-        <v>35</v>
+        <v>58</v>
       </c>
       <c r="O276" t="n">
-        <v>35</v>
+        <v>58</v>
       </c>
       <c r="P276" t="n">
         <v>0</v>
@@ -21699,22 +21699,22 @@
       </c>
       <c r="V276" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11497.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11500.jpg</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="n">
-        <v>11499</v>
+        <v>11502</v>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>78</t>
+          <t>2808</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>TEMPERO BAIANO PO</t>
+          <t>TEMPERO ANA MARIA</t>
         </is>
       </c>
       <c r="F277" t="inlineStr">
@@ -21750,10 +21750,10 @@
         </is>
       </c>
       <c r="N277" t="n">
-        <v>13</v>
+        <v>38</v>
       </c>
       <c r="O277" t="n">
-        <v>13</v>
+        <v>38</v>
       </c>
       <c r="P277" t="n">
         <v>0</v>
@@ -21776,22 +21776,22 @@
       </c>
       <c r="V277" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11499.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11502.jpg</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="n">
-        <v>11500</v>
+        <v>11523</v>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>79</t>
+          <t>58</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>TEMPERO BAIANO GRAO</t>
+          <t>SALSA DESIDRATADA</t>
         </is>
       </c>
       <c r="F278" t="inlineStr">
@@ -21827,10 +21827,10 @@
         </is>
       </c>
       <c r="N278" t="n">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="O278" t="n">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="P278" t="n">
         <v>0</v>
@@ -21853,22 +21853,22 @@
       </c>
       <c r="V278" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11500.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11523.jpg</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="n">
-        <v>11502</v>
+        <v>11563</v>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>2808</t>
+          <t>84</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>TEMPERO ANA MARIA</t>
+          <t>PIMENTA SIRIA PO (JAMAICA)</t>
         </is>
       </c>
       <c r="F279" t="inlineStr">
@@ -21904,10 +21904,10 @@
         </is>
       </c>
       <c r="N279" t="n">
-        <v>38</v>
+        <v>165</v>
       </c>
       <c r="O279" t="n">
-        <v>38</v>
+        <v>165</v>
       </c>
       <c r="P279" t="n">
         <v>0</v>
@@ -21930,22 +21930,22 @@
       </c>
       <c r="V279" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11502.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11563.jpg</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="n">
-        <v>11523</v>
+        <v>11565</v>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>4273</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>SALSA DESIDRATADA</t>
+          <t>PIMENTA SIRIA GRAO (JAMAICA)</t>
         </is>
       </c>
       <c r="F280" t="inlineStr">
@@ -21981,10 +21981,10 @@
         </is>
       </c>
       <c r="N280" t="n">
-        <v>48</v>
+        <v>220</v>
       </c>
       <c r="O280" t="n">
-        <v>48</v>
+        <v>220</v>
       </c>
       <c r="P280" t="n">
         <v>0</v>
@@ -22007,22 +22007,22 @@
       </c>
       <c r="V280" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11523.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11565.jpg</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="n">
-        <v>11563</v>
+        <v>11567</v>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>99</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>PIMENTA SIRIA PO (JAMAICA)</t>
+          <t>PIMENTA ROSA</t>
         </is>
       </c>
       <c r="F281" t="inlineStr">
@@ -22058,10 +22058,10 @@
         </is>
       </c>
       <c r="N281" t="n">
-        <v>165</v>
+        <v>108</v>
       </c>
       <c r="O281" t="n">
-        <v>165</v>
+        <v>108</v>
       </c>
       <c r="P281" t="n">
         <v>0</v>
@@ -22084,22 +22084,22 @@
       </c>
       <c r="V281" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11563.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11567.jpg</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="n">
-        <v>11565</v>
+        <v>11568</v>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>4273</t>
+          <t>77</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>PIMENTA SIRIA GRAO (JAMAICA)</t>
+          <t>PIMENTA DO REINO PRETA PO</t>
         </is>
       </c>
       <c r="F282" t="inlineStr">
@@ -22135,10 +22135,10 @@
         </is>
       </c>
       <c r="N282" t="n">
-        <v>220</v>
+        <v>68</v>
       </c>
       <c r="O282" t="n">
-        <v>220</v>
+        <v>68</v>
       </c>
       <c r="P282" t="n">
         <v>0</v>
@@ -22161,22 +22161,22 @@
       </c>
       <c r="V282" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11565.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11568.jpg</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="n">
-        <v>11567</v>
+        <v>11569</v>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>53</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>PIMENTA ROSA</t>
+          <t>PIMENTA DO REINO  PRETA  GRAO</t>
         </is>
       </c>
       <c r="F283" t="inlineStr">
@@ -22212,10 +22212,10 @@
         </is>
       </c>
       <c r="N283" t="n">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="O283" t="n">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="P283" t="n">
         <v>0</v>
@@ -22238,22 +22238,22 @@
       </c>
       <c r="V283" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11567.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11569.jpg</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="n">
-        <v>11568</v>
+        <v>11570</v>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>3154</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>PIMENTA DO REINO PRETA PO</t>
+          <t>PIMENTA DO REINO BRANCA EM PO</t>
         </is>
       </c>
       <c r="F284" t="inlineStr">
@@ -22289,10 +22289,10 @@
         </is>
       </c>
       <c r="N284" t="n">
-        <v>68</v>
+        <v>225</v>
       </c>
       <c r="O284" t="n">
-        <v>68</v>
+        <v>225</v>
       </c>
       <c r="P284" t="n">
         <v>0</v>
@@ -22315,22 +22315,22 @@
       </c>
       <c r="V284" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11568.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11570.jpg</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="n">
-        <v>11569</v>
+        <v>11571</v>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>3458</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>PIMENTA DO REINO  PRETA  GRAO</t>
+          <t>PIMENTA CHILLI</t>
         </is>
       </c>
       <c r="F285" t="inlineStr">
@@ -22366,10 +22366,10 @@
         </is>
       </c>
       <c r="N285" t="n">
-        <v>95</v>
+        <v>75</v>
       </c>
       <c r="O285" t="n">
-        <v>95</v>
+        <v>75</v>
       </c>
       <c r="P285" t="n">
         <v>0</v>
@@ -22392,22 +22392,22 @@
       </c>
       <c r="V285" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11569.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11571.png</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="n">
-        <v>11570</v>
+        <v>11572</v>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>3154</t>
+          <t>59</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>PIMENTA DO REINO BRANCA EM PO</t>
+          <t>PIMENTA CALABRESA FLOCOS</t>
         </is>
       </c>
       <c r="F286" t="inlineStr">
@@ -22443,10 +22443,10 @@
         </is>
       </c>
       <c r="N286" t="n">
-        <v>225</v>
+        <v>40</v>
       </c>
       <c r="O286" t="n">
-        <v>225</v>
+        <v>40</v>
       </c>
       <c r="P286" t="n">
         <v>0</v>
@@ -22469,22 +22469,22 @@
       </c>
       <c r="V286" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11570.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11572.webp</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="n">
-        <v>11571</v>
+        <v>11573</v>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>3458</t>
+          <t>607</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>PIMENTA CHILLI</t>
+          <t>PIMENTA CAYENA</t>
         </is>
       </c>
       <c r="F287" t="inlineStr">
@@ -22520,10 +22520,10 @@
         </is>
       </c>
       <c r="N287" t="n">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="O287" t="n">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="P287" t="n">
         <v>0</v>
@@ -22546,22 +22546,22 @@
       </c>
       <c r="V287" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11571.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11573.jpg</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="n">
-        <v>11572</v>
+        <v>11584</v>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>3347</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>PIMENTA CALABRESA FLOCOS</t>
+          <t>PAPRICA PICANTE</t>
         </is>
       </c>
       <c r="F288" t="inlineStr">
@@ -22597,10 +22597,10 @@
         </is>
       </c>
       <c r="N288" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O288" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="P288" t="n">
         <v>0</v>
@@ -22623,22 +22623,22 @@
       </c>
       <c r="V288" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11572.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11584.jpg</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="n">
-        <v>11573</v>
+        <v>11586</v>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>607</t>
+          <t>3348</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>PIMENTA CAYENA</t>
+          <t>PAPRICA DOCE</t>
         </is>
       </c>
       <c r="F289" t="inlineStr">
@@ -22674,10 +22674,10 @@
         </is>
       </c>
       <c r="N289" t="n">
-        <v>68</v>
+        <v>30</v>
       </c>
       <c r="O289" t="n">
-        <v>68</v>
+        <v>30</v>
       </c>
       <c r="P289" t="n">
         <v>0</v>
@@ -22700,22 +22700,22 @@
       </c>
       <c r="V289" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11573.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11586.jpg</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="n">
-        <v>11584</v>
+        <v>11588</v>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>3347</t>
+          <t>3172</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>PAPRICA PICANTE</t>
+          <t>PAPRICA DEFUMADA</t>
         </is>
       </c>
       <c r="F290" t="inlineStr">
@@ -22777,22 +22777,22 @@
       </c>
       <c r="V290" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11584.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11588.jpg</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="n">
-        <v>11586</v>
+        <v>11592</v>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>3348</t>
+          <t>56</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>PAPRICA DOCE</t>
+          <t>OREGANO</t>
         </is>
       </c>
       <c r="F291" t="inlineStr">
@@ -22828,10 +22828,10 @@
         </is>
       </c>
       <c r="N291" t="n">
-        <v>30</v>
+        <v>53</v>
       </c>
       <c r="O291" t="n">
-        <v>30</v>
+        <v>53</v>
       </c>
       <c r="P291" t="n">
         <v>0</v>
@@ -22854,22 +22854,22 @@
       </c>
       <c r="V291" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11586.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11592.jpg</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="n">
-        <v>11588</v>
+        <v>11602</v>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>3172</t>
+          <t>1725</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>PAPRICA DEFUMADA</t>
+          <t>NOZ MOSCADA PO</t>
         </is>
       </c>
       <c r="F292" t="inlineStr">
@@ -22905,10 +22905,10 @@
         </is>
       </c>
       <c r="N292" t="n">
-        <v>30</v>
+        <v>160</v>
       </c>
       <c r="O292" t="n">
-        <v>30</v>
+        <v>160</v>
       </c>
       <c r="P292" t="n">
         <v>0</v>
@@ -22931,22 +22931,22 @@
       </c>
       <c r="V292" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11588.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11602.jpg</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" t="n">
-        <v>11592</v>
+        <v>11607</v>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>3566</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>OREGANO</t>
+          <t>MOSTARDA PO PURA</t>
         </is>
       </c>
       <c r="F293" t="inlineStr">
@@ -22982,10 +22982,10 @@
         </is>
       </c>
       <c r="N293" t="n">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="O293" t="n">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="P293" t="n">
         <v>0</v>
@@ -23008,22 +23008,22 @@
       </c>
       <c r="V293" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11592.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11607.png</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" t="n">
-        <v>11602</v>
+        <v>11608</v>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>1725</t>
+          <t>3411</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>NOZ MOSCADA PO</t>
+          <t>MOSTARDA GRAO</t>
         </is>
       </c>
       <c r="F294" t="inlineStr">
@@ -23059,10 +23059,10 @@
         </is>
       </c>
       <c r="N294" t="n">
-        <v>160</v>
+        <v>45</v>
       </c>
       <c r="O294" t="n">
-        <v>160</v>
+        <v>45</v>
       </c>
       <c r="P294" t="n">
         <v>0</v>
@@ -23085,22 +23085,22 @@
       </c>
       <c r="V294" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11602.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11608.jpg</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" t="n">
-        <v>11607</v>
+        <v>11629</v>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>3566</t>
+          <t>66</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>MOSTARDA PO PURA</t>
+          <t>MANJERONA DESIDRATADO</t>
         </is>
       </c>
       <c r="F295" t="inlineStr">
@@ -23136,10 +23136,10 @@
         </is>
       </c>
       <c r="N295" t="n">
-        <v>58</v>
+        <v>30</v>
       </c>
       <c r="O295" t="n">
-        <v>58</v>
+        <v>30</v>
       </c>
       <c r="P295" t="n">
         <v>0</v>
@@ -23162,22 +23162,22 @@
       </c>
       <c r="V295" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11607.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11629.jpg</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" t="n">
-        <v>11608</v>
+        <v>11630</v>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>3411</t>
+          <t>65</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>MOSTARDA GRAO</t>
+          <t>MANJERICAO DESIDRATADO</t>
         </is>
       </c>
       <c r="F296" t="inlineStr">
@@ -23213,10 +23213,10 @@
         </is>
       </c>
       <c r="N296" t="n">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="O296" t="n">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="P296" t="n">
         <v>0</v>
@@ -23239,22 +23239,22 @@
       </c>
       <c r="V296" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11608.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11630.png</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" t="n">
-        <v>11629</v>
+        <v>11642</v>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>80</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>MANJERONA DESIDRATADO</t>
+          <t>LOURO EM PO</t>
         </is>
       </c>
       <c r="F297" t="inlineStr">
@@ -23290,10 +23290,10 @@
         </is>
       </c>
       <c r="N297" t="n">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="O297" t="n">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="P297" t="n">
         <v>0</v>
@@ -23316,22 +23316,22 @@
       </c>
       <c r="V297" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11629.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11642.png</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" t="n">
-        <v>11630</v>
+        <v>11643</v>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>65</t>
+          <t>811</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>MANJERICAO DESIDRATADO</t>
+          <t>LOURO EM FOLHA</t>
         </is>
       </c>
       <c r="F298" t="inlineStr">
@@ -23367,10 +23367,10 @@
         </is>
       </c>
       <c r="N298" t="n">
-        <v>28</v>
+        <v>75</v>
       </c>
       <c r="O298" t="n">
-        <v>28</v>
+        <v>75</v>
       </c>
       <c r="P298" t="n">
         <v>0</v>
@@ -23393,22 +23393,22 @@
       </c>
       <c r="V298" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11630.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11643.webp</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" t="n">
-        <v>11642</v>
+        <v>11647</v>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>5006</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>LOURO EM PO</t>
+          <t>LEMON PEPPER 0% SODIO</t>
         </is>
       </c>
       <c r="F299" t="inlineStr">
@@ -23444,10 +23444,10 @@
         </is>
       </c>
       <c r="N299" t="n">
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="O299" t="n">
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="P299" t="n">
         <v>0</v>
@@ -23470,22 +23470,22 @@
       </c>
       <c r="V299" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11642.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11647.jpg</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" t="n">
-        <v>11643</v>
+        <v>11655</v>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>811</t>
+          <t>3346</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>LOURO EM FOLHA</t>
+          <t>LEMON PEPPER</t>
         </is>
       </c>
       <c r="F300" t="inlineStr">
@@ -23521,10 +23521,10 @@
         </is>
       </c>
       <c r="N300" t="n">
-        <v>75</v>
+        <v>45</v>
       </c>
       <c r="O300" t="n">
-        <v>75</v>
+        <v>45</v>
       </c>
       <c r="P300" t="n">
         <v>0</v>
@@ -23547,22 +23547,22 @@
       </c>
       <c r="V300" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11643.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11655.jpg</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" t="n">
-        <v>11647</v>
+        <v>11717</v>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>5006</t>
+          <t>3503</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>LEMON PEPPER 0% SODIO</t>
+          <t>FUMACA EM PO</t>
         </is>
       </c>
       <c r="F301" t="inlineStr">
@@ -23598,10 +23598,10 @@
         </is>
       </c>
       <c r="N301" t="n">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="O301" t="n">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="P301" t="n">
         <v>0</v>
@@ -23624,22 +23624,22 @@
       </c>
       <c r="V301" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11647.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11717.jpg</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" t="n">
-        <v>11655</v>
+        <v>11806</v>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>3346</t>
+          <t>96</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>LEMON PEPPER</t>
+          <t>ERVAS FINAS</t>
         </is>
       </c>
       <c r="F302" t="inlineStr">
@@ -23675,10 +23675,10 @@
         </is>
       </c>
       <c r="N302" t="n">
-        <v>45</v>
+        <v>85</v>
       </c>
       <c r="O302" t="n">
-        <v>45</v>
+        <v>85</v>
       </c>
       <c r="P302" t="n">
         <v>0</v>
@@ -23701,22 +23701,22 @@
       </c>
       <c r="V302" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11655.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11806.jpg</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" t="n">
-        <v>11717</v>
+        <v>11818</v>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>3503</t>
+          <t>3446</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>FUMACA EM PO</t>
+          <t>ENDRO</t>
         </is>
       </c>
       <c r="F303" t="inlineStr">
@@ -23752,10 +23752,10 @@
         </is>
       </c>
       <c r="N303" t="n">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="O303" t="n">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="P303" t="n">
         <v>0</v>
@@ -23778,22 +23778,22 @@
       </c>
       <c r="V303" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11717.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11818.jpg</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" t="n">
-        <v>11806</v>
+        <v>11822</v>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>96</t>
+          <t>2809</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>ERVAS FINAS</t>
+          <t>EDU GUEDES</t>
         </is>
       </c>
       <c r="F304" t="inlineStr">
@@ -23829,10 +23829,10 @@
         </is>
       </c>
       <c r="N304" t="n">
-        <v>85</v>
+        <v>50</v>
       </c>
       <c r="O304" t="n">
-        <v>85</v>
+        <v>50</v>
       </c>
       <c r="P304" t="n">
         <v>0</v>
@@ -23855,22 +23855,22 @@
       </c>
       <c r="V304" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11806.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11822.jpg</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" t="n">
-        <v>11818</v>
+        <v>11830</v>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>3446</t>
+          <t>3402</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>ENDRO</t>
+          <t>CURRY</t>
         </is>
       </c>
       <c r="F305" t="inlineStr">
@@ -23906,10 +23906,10 @@
         </is>
       </c>
       <c r="N305" t="n">
-        <v>58</v>
+        <v>20</v>
       </c>
       <c r="O305" t="n">
-        <v>58</v>
+        <v>20</v>
       </c>
       <c r="P305" t="n">
         <v>0</v>
@@ -23932,22 +23932,22 @@
       </c>
       <c r="V305" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11818.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11830.jpg</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" t="n">
-        <v>11822</v>
+        <v>11833</v>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>2809</t>
+          <t>89</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>EDU GUEDES</t>
+          <t>CRAVO MOIDO</t>
         </is>
       </c>
       <c r="F306" t="inlineStr">
@@ -23983,10 +23983,10 @@
         </is>
       </c>
       <c r="N306" t="n">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="O306" t="n">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="P306" t="n">
         <v>0</v>
@@ -24009,22 +24009,22 @@
       </c>
       <c r="V306" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11822.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11833.jpg</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" t="n">
-        <v>11830</v>
+        <v>11834</v>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>3402</t>
+          <t>90</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>CURRY</t>
+          <t>CRAVO GRAO</t>
         </is>
       </c>
       <c r="F307" t="inlineStr">
@@ -24060,10 +24060,10 @@
         </is>
       </c>
       <c r="N307" t="n">
-        <v>20</v>
+        <v>110</v>
       </c>
       <c r="O307" t="n">
-        <v>20</v>
+        <v>110</v>
       </c>
       <c r="P307" t="n">
         <v>0</v>
@@ -24086,22 +24086,22 @@
       </c>
       <c r="V307" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11830.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11834.jpg</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" t="n">
-        <v>11833</v>
+        <v>11838</v>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>89</t>
+          <t>3761</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>CRAVO MOIDO</t>
+          <t>COMINHO PO PURO</t>
         </is>
       </c>
       <c r="F308" t="inlineStr">
@@ -24137,10 +24137,10 @@
         </is>
       </c>
       <c r="N308" t="n">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="O308" t="n">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="P308" t="n">
         <v>0</v>
@@ -24163,22 +24163,22 @@
       </c>
       <c r="V308" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11833.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11838.png</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" t="n">
-        <v>11834</v>
+        <v>11839</v>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>54</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>CRAVO GRAO</t>
+          <t>COMINHO GRAO 99%</t>
         </is>
       </c>
       <c r="F309" t="inlineStr">
@@ -24214,10 +24214,10 @@
         </is>
       </c>
       <c r="N309" t="n">
-        <v>110</v>
+        <v>48</v>
       </c>
       <c r="O309" t="n">
-        <v>110</v>
+        <v>48</v>
       </c>
       <c r="P309" t="n">
         <v>0</v>
@@ -24240,22 +24240,22 @@
       </c>
       <c r="V309" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11834.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11839.png</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="n">
-        <v>11838</v>
+        <v>11840</v>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>3761</t>
+          <t>571</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>COMINHO PO PURO</t>
+          <t>COLORAU</t>
         </is>
       </c>
       <c r="F310" t="inlineStr">
@@ -24291,10 +24291,10 @@
         </is>
       </c>
       <c r="N310" t="n">
-        <v>65</v>
+        <v>20</v>
       </c>
       <c r="O310" t="n">
-        <v>65</v>
+        <v>20</v>
       </c>
       <c r="P310" t="n">
         <v>0</v>
@@ -24317,22 +24317,22 @@
       </c>
       <c r="V310" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11838.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11840.jpg</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="n">
-        <v>11839</v>
+        <v>11843</v>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>54</t>
+          <t>55</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>COMINHO GRAO 99%</t>
+          <t>COENTRO GRAO</t>
         </is>
       </c>
       <c r="F311" t="inlineStr">
@@ -24368,10 +24368,10 @@
         </is>
       </c>
       <c r="N311" t="n">
-        <v>48</v>
+        <v>17.5</v>
       </c>
       <c r="O311" t="n">
-        <v>48</v>
+        <v>17.5</v>
       </c>
       <c r="P311" t="n">
         <v>0</v>
@@ -24394,22 +24394,22 @@
       </c>
       <c r="V311" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11839.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11843.jpg</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="n">
-        <v>11840</v>
+        <v>11844</v>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>571</t>
+          <t>5161</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>COLORAU</t>
+          <t>COENTRO FOLHAS</t>
         </is>
       </c>
       <c r="F312" t="inlineStr">
@@ -24445,10 +24445,10 @@
         </is>
       </c>
       <c r="N312" t="n">
-        <v>20</v>
+        <v>64</v>
       </c>
       <c r="O312" t="n">
-        <v>20</v>
+        <v>64</v>
       </c>
       <c r="P312" t="n">
         <v>0</v>
@@ -24471,22 +24471,22 @@
       </c>
       <c r="V312" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11840.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11844.webp</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="n">
-        <v>11843</v>
+        <v>11845</v>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>3947</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>COENTRO GRAO</t>
+          <t>COENTRO EM PO</t>
         </is>
       </c>
       <c r="F313" t="inlineStr">
@@ -24522,10 +24522,10 @@
         </is>
       </c>
       <c r="N313" t="n">
-        <v>17.5</v>
+        <v>19</v>
       </c>
       <c r="O313" t="n">
-        <v>17.5</v>
+        <v>19</v>
       </c>
       <c r="P313" t="n">
         <v>0</v>
@@ -24548,22 +24548,22 @@
       </c>
       <c r="V313" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11843.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11845.png</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="n">
-        <v>11844</v>
+        <v>11863</v>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>5161</t>
+          <t>404</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>COENTRO FOLHAS</t>
+          <t>CHIMICHURRI SEM PIMENTA</t>
         </is>
       </c>
       <c r="F314" t="inlineStr">
@@ -24599,10 +24599,10 @@
         </is>
       </c>
       <c r="N314" t="n">
-        <v>64</v>
+        <v>50</v>
       </c>
       <c r="O314" t="n">
-        <v>64</v>
+        <v>50</v>
       </c>
       <c r="P314" t="n">
         <v>0</v>
@@ -24625,22 +24625,22 @@
       </c>
       <c r="V314" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11844.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11863.jpg</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="n">
-        <v>11845</v>
+        <v>11864</v>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>3947</t>
+          <t>3690</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>COENTRO EM PO</t>
+          <t>CHIMICHURRI COM PIMENTA</t>
         </is>
       </c>
       <c r="F315" t="inlineStr">
@@ -24676,10 +24676,10 @@
         </is>
       </c>
       <c r="N315" t="n">
-        <v>19</v>
+        <v>50</v>
       </c>
       <c r="O315" t="n">
-        <v>19</v>
+        <v>50</v>
       </c>
       <c r="P315" t="n">
         <v>0</v>
@@ -24702,22 +24702,22 @@
       </c>
       <c r="V315" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11845.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11864.webp</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="n">
-        <v>11863</v>
+        <v>11874</v>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>404</t>
+          <t>63</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>CHIMICHURRI SEM PIMENTA</t>
+          <t>CEBOLINHA DESIDRATADA</t>
         </is>
       </c>
       <c r="F316" t="inlineStr">
@@ -24753,10 +24753,10 @@
         </is>
       </c>
       <c r="N316" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="O316" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="P316" t="n">
         <v>0</v>
@@ -24779,22 +24779,22 @@
       </c>
       <c r="V316" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11863.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11874.webp</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="n">
-        <v>11864</v>
+        <v>11875</v>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>3690</t>
+          <t>3295</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>CHIMICHURRI COM PIMENTA</t>
+          <t>CEBOLA, ALHO E SALSA</t>
         </is>
       </c>
       <c r="F317" t="inlineStr">
@@ -24830,10 +24830,10 @@
         </is>
       </c>
       <c r="N317" t="n">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="O317" t="n">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="P317" t="n">
         <v>0</v>
@@ -24856,22 +24856,22 @@
       </c>
       <c r="V317" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11864.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11875.jpg</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="n">
-        <v>11874</v>
+        <v>11877</v>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>63</t>
+          <t>62</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>CEBOLINHA DESIDRATADA</t>
+          <t>CEBOLA FLOCOS</t>
         </is>
       </c>
       <c r="F318" t="inlineStr">
@@ -24907,10 +24907,10 @@
         </is>
       </c>
       <c r="N318" t="n">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="O318" t="n">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="P318" t="n">
         <v>0</v>
@@ -24933,22 +24933,22 @@
       </c>
       <c r="V318" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11874.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11877.jpg</t>
         </is>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="n">
-        <v>11875</v>
+        <v>11879</v>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>3295</t>
+          <t>982</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>CEBOLA, ALHO E SALSA</t>
+          <t>CEBOLA EM PO</t>
         </is>
       </c>
       <c r="F319" t="inlineStr">
@@ -24984,10 +24984,10 @@
         </is>
       </c>
       <c r="N319" t="n">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="O319" t="n">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="P319" t="n">
         <v>0</v>
@@ -25010,22 +25010,22 @@
       </c>
       <c r="V319" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11875.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11879.jpg</t>
         </is>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="n">
-        <v>11877</v>
+        <v>11909</v>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>3334</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>CEBOLA FLOCOS</t>
+          <t>CARDAMOMO SEMENTES</t>
         </is>
       </c>
       <c r="F320" t="inlineStr">
@@ -25061,10 +25061,10 @@
         </is>
       </c>
       <c r="N320" t="n">
-        <v>53</v>
+        <v>680</v>
       </c>
       <c r="O320" t="n">
-        <v>53</v>
+        <v>680</v>
       </c>
       <c r="P320" t="n">
         <v>0</v>
@@ -25087,22 +25087,22 @@
       </c>
       <c r="V320" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11877.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11909.jpg</t>
         </is>
       </c>
     </row>
     <row r="321">
       <c r="A321" t="n">
-        <v>11879</v>
+        <v>11910</v>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>982</t>
+          <t>3837</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>CEBOLA EM PO</t>
+          <t>CARDAMOMO PO</t>
         </is>
       </c>
       <c r="F321" t="inlineStr">
@@ -25138,10 +25138,10 @@
         </is>
       </c>
       <c r="N321" t="n">
-        <v>45</v>
+        <v>680</v>
       </c>
       <c r="O321" t="n">
-        <v>45</v>
+        <v>680</v>
       </c>
       <c r="P321" t="n">
         <v>0</v>
@@ -25164,22 +25164,22 @@
       </c>
       <c r="V321" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11879.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11910.png</t>
         </is>
       </c>
     </row>
     <row r="322">
       <c r="A322" t="n">
-        <v>11909</v>
+        <v>11913</v>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>3334</t>
+          <t>87</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>CARDAMOMO SEMENTES</t>
+          <t>CANELA EM PO PURA</t>
         </is>
       </c>
       <c r="F322" t="inlineStr">
@@ -25215,10 +25215,10 @@
         </is>
       </c>
       <c r="N322" t="n">
-        <v>680</v>
+        <v>35</v>
       </c>
       <c r="O322" t="n">
-        <v>680</v>
+        <v>35</v>
       </c>
       <c r="P322" t="n">
         <v>0</v>
@@ -25241,22 +25241,22 @@
       </c>
       <c r="V322" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11909.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11913.jpg</t>
         </is>
       </c>
     </row>
     <row r="323">
       <c r="A323" t="n">
-        <v>11910</v>
+        <v>11931</v>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>3837</t>
+          <t>1571</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>CARDAMOMO PO</t>
+          <t>BICARBONATO DE SODIO</t>
         </is>
       </c>
       <c r="F323" t="inlineStr">
@@ -25292,10 +25292,10 @@
         </is>
       </c>
       <c r="N323" t="n">
-        <v>680</v>
+        <v>10.5</v>
       </c>
       <c r="O323" t="n">
-        <v>680</v>
+        <v>10.5</v>
       </c>
       <c r="P323" t="n">
         <v>0</v>
@@ -25318,22 +25318,22 @@
       </c>
       <c r="V323" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11910.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11931.webp</t>
         </is>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="n">
-        <v>11913</v>
+        <v>12004</v>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>321</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>CANELA EM PO PURA</t>
+          <t>ALHO ROXO</t>
         </is>
       </c>
       <c r="F324" t="inlineStr">
@@ -25369,10 +25369,10 @@
         </is>
       </c>
       <c r="N324" t="n">
-        <v>35</v>
+        <v>49</v>
       </c>
       <c r="O324" t="n">
-        <v>35</v>
+        <v>49</v>
       </c>
       <c r="P324" t="n">
         <v>0</v>
@@ -25395,22 +25395,22 @@
       </c>
       <c r="V324" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11913.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12004.jpg</t>
         </is>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="n">
-        <v>11931</v>
+        <v>12006</v>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>1571</t>
+          <t>61</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>BICARBONATO DE SODIO</t>
+          <t>ALHO LAMINADO DESIDRATADO</t>
         </is>
       </c>
       <c r="F325" t="inlineStr">
@@ -25446,10 +25446,10 @@
         </is>
       </c>
       <c r="N325" t="n">
-        <v>10.5</v>
+        <v>85</v>
       </c>
       <c r="O325" t="n">
-        <v>10.5</v>
+        <v>85</v>
       </c>
       <c r="P325" t="n">
         <v>0</v>
@@ -25472,22 +25472,22 @@
       </c>
       <c r="V325" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11931.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12006.webp</t>
         </is>
       </c>
     </row>
     <row r="326">
       <c r="A326" t="n">
-        <v>12004</v>
+        <v>12008</v>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>321</t>
+          <t>60</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>ALHO ROXO</t>
+          <t>ALHO GRANULADO</t>
         </is>
       </c>
       <c r="F326" t="inlineStr">
@@ -25549,22 +25549,22 @@
       </c>
       <c r="V326" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12004.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12008.webp</t>
         </is>
       </c>
     </row>
     <row r="327">
       <c r="A327" t="n">
-        <v>12006</v>
+        <v>12010</v>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>61</t>
+          <t>422</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>ALHO LAMINADO DESIDRATADO</t>
+          <t>ALHO FRITO</t>
         </is>
       </c>
       <c r="F327" t="inlineStr">
@@ -25600,10 +25600,10 @@
         </is>
       </c>
       <c r="N327" t="n">
-        <v>85</v>
+        <v>48</v>
       </c>
       <c r="O327" t="n">
-        <v>85</v>
+        <v>48</v>
       </c>
       <c r="P327" t="n">
         <v>0</v>
@@ -25626,22 +25626,22 @@
       </c>
       <c r="V327" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12006.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12010.jpg</t>
         </is>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="n">
-        <v>12008</v>
+        <v>12011</v>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>3350</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>ALHO GRANULADO</t>
+          <t>ALHO EM PO 100% PURO</t>
         </is>
       </c>
       <c r="F328" t="inlineStr">
@@ -25677,10 +25677,10 @@
         </is>
       </c>
       <c r="N328" t="n">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="O328" t="n">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="P328" t="n">
         <v>0</v>
@@ -25703,22 +25703,22 @@
       </c>
       <c r="V328" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12008.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12011.jpg</t>
         </is>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="n">
-        <v>12010</v>
+        <v>12019</v>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>422</t>
+          <t>67</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>ALHO FRITO</t>
+          <t>ALECRIM</t>
         </is>
       </c>
       <c r="F329" t="inlineStr">
@@ -25754,10 +25754,10 @@
         </is>
       </c>
       <c r="N329" t="n">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="O329" t="n">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="P329" t="n">
         <v>0</v>
@@ -25780,22 +25780,22 @@
       </c>
       <c r="V329" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12010.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12019.jpg</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="n">
-        <v>12011</v>
+        <v>12023</v>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>3350</t>
+          <t>4139</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>ALHO EM PO 100% PURO</t>
+          <t>AIPO</t>
         </is>
       </c>
       <c r="F330" t="inlineStr">
@@ -25831,10 +25831,10 @@
         </is>
       </c>
       <c r="N330" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="O330" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="P330" t="n">
         <v>0</v>
@@ -25857,22 +25857,22 @@
       </c>
       <c r="V330" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12011.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12023.jpg</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" t="n">
-        <v>12019</v>
+        <v>12031</v>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>1665</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>ALECRIM</t>
+          <t>ACAFRAO NACIONAL</t>
         </is>
       </c>
       <c r="F331" t="inlineStr">
@@ -25908,10 +25908,10 @@
         </is>
       </c>
       <c r="N331" t="n">
-        <v>40</v>
+        <v>105</v>
       </c>
       <c r="O331" t="n">
-        <v>40</v>
+        <v>105</v>
       </c>
       <c r="P331" t="n">
         <v>0</v>
@@ -25934,22 +25934,22 @@
       </c>
       <c r="V331" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12019.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12031.jpg</t>
         </is>
       </c>
     </row>
     <row r="332">
       <c r="A332" t="n">
-        <v>12023</v>
+        <v>12080</v>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>4139</t>
+          <t>3234</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>AIPO</t>
+          <t>CALDO DE GALINHA</t>
         </is>
       </c>
       <c r="F332" t="inlineStr">
@@ -25985,10 +25985,10 @@
         </is>
       </c>
       <c r="N332" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="O332" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="P332" t="n">
         <v>0</v>
@@ -26011,22 +26011,22 @@
       </c>
       <c r="V332" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12023.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12080.jpg</t>
         </is>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="n">
-        <v>12031</v>
+        <v>12098</v>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>1665</t>
+          <t>3242</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>ACAFRAO NACIONAL</t>
+          <t>CALDO DE LEGUMES</t>
         </is>
       </c>
       <c r="F333" t="inlineStr">
@@ -26062,10 +26062,10 @@
         </is>
       </c>
       <c r="N333" t="n">
-        <v>105</v>
+        <v>0</v>
       </c>
       <c r="O333" t="n">
-        <v>105</v>
+        <v>0</v>
       </c>
       <c r="P333" t="n">
         <v>0</v>
@@ -26088,22 +26088,22 @@
       </c>
       <c r="V333" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12031.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12098.jpg</t>
         </is>
       </c>
     </row>
     <row r="334">
       <c r="A334" t="n">
-        <v>12080</v>
+        <v>12105</v>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>3234</t>
+          <t>199</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>CALDO DE GALINHA</t>
+          <t>EDU GUEDES</t>
         </is>
       </c>
       <c r="F334" t="inlineStr">
@@ -26139,10 +26139,10 @@
         </is>
       </c>
       <c r="N334" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="O334" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="P334" t="n">
         <v>0</v>
@@ -26165,22 +26165,22 @@
       </c>
       <c r="V334" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12080.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12105.jpg</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="n">
-        <v>12098</v>
+        <v>12106</v>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>3242</t>
+          <t>200</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>CALDO DE LEGUMES</t>
+          <t>ANA MARIA</t>
         </is>
       </c>
       <c r="F335" t="inlineStr">
@@ -26216,10 +26216,10 @@
         </is>
       </c>
       <c r="N335" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="O335" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="P335" t="n">
         <v>0</v>
@@ -26242,22 +26242,22 @@
       </c>
       <c r="V335" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12098.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12106.jpg</t>
         </is>
       </c>
     </row>
     <row r="336">
       <c r="A336" t="n">
-        <v>12105</v>
+        <v>12107</v>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>199</t>
+          <t>201</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>EDU GUEDES</t>
+          <t>CEBOLA, ALHO E SALSA</t>
         </is>
       </c>
       <c r="F336" t="inlineStr">
@@ -26293,10 +26293,10 @@
         </is>
       </c>
       <c r="N336" t="n">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="O336" t="n">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="P336" t="n">
         <v>0</v>
@@ -26319,22 +26319,22 @@
       </c>
       <c r="V336" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12105.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12107.jpg</t>
         </is>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="n">
-        <v>12106</v>
+        <v>12108</v>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>202</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>ANA MARIA</t>
+          <t>CHIMICHURRI SEM PIMENTA</t>
         </is>
       </c>
       <c r="F337" t="inlineStr">
@@ -26370,10 +26370,10 @@
         </is>
       </c>
       <c r="N337" t="n">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="O337" t="n">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="P337" t="n">
         <v>0</v>
@@ -26396,22 +26396,22 @@
       </c>
       <c r="V337" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12106.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12108.jpg</t>
         </is>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="n">
-        <v>12107</v>
+        <v>12109</v>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>201</t>
+          <t>203</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>CEBOLA, ALHO E SALSA</t>
+          <t>CHIMICHURRI COM PIMENTA</t>
         </is>
       </c>
       <c r="F338" t="inlineStr">
@@ -26447,10 +26447,10 @@
         </is>
       </c>
       <c r="N338" t="n">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="O338" t="n">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="P338" t="n">
         <v>0</v>
@@ -26473,22 +26473,22 @@
       </c>
       <c r="V338" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12107.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12109.webp</t>
         </is>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="n">
-        <v>12108</v>
+        <v>12096</v>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>202</t>
+          <t>1209</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>CHIMICHURRI SEM PIMENTA</t>
+          <t>PEGA MARIDO FIT</t>
         </is>
       </c>
       <c r="F339" t="inlineStr">
@@ -26524,10 +26524,10 @@
         </is>
       </c>
       <c r="N339" t="n">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="O339" t="n">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="P339" t="n">
         <v>0</v>
@@ -26550,22 +26550,22 @@
       </c>
       <c r="V339" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12108.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12096.jpg</t>
         </is>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="n">
-        <v>12109</v>
+        <v>12097</v>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>203</t>
+          <t>1299</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>CHIMICHURRI COM PIMENTA</t>
+          <t>EDU GUEDES FIT</t>
         </is>
       </c>
       <c r="F340" t="inlineStr">
@@ -26627,22 +26627,22 @@
       </c>
       <c r="V340" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12109.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12097.jpg</t>
         </is>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="n">
-        <v>12096</v>
+        <v>12119</v>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>1209</t>
+          <t>3146</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>PEGA MARIDO FIT</t>
+          <t>CEBOLA GRANULADA</t>
         </is>
       </c>
       <c r="F341" t="inlineStr">
@@ -26678,10 +26678,10 @@
         </is>
       </c>
       <c r="N341" t="n">
-        <v>59</v>
+        <v>42</v>
       </c>
       <c r="O341" t="n">
-        <v>59</v>
+        <v>42</v>
       </c>
       <c r="P341" t="n">
         <v>0</v>
@@ -26704,22 +26704,22 @@
       </c>
       <c r="V341" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12096.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12119.jpg</t>
         </is>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="n">
-        <v>12097</v>
+        <v>12115</v>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>1299</t>
+          <t>209</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>EDU GUEDES FIT</t>
+          <t>LEMON PEPPER C/ GLUTAMATO</t>
         </is>
       </c>
       <c r="F342" t="inlineStr">
@@ -26755,10 +26755,10 @@
         </is>
       </c>
       <c r="N342" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="O342" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="P342" t="n">
         <v>0</v>
@@ -26781,22 +26781,22 @@
       </c>
       <c r="V342" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12097.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12115.png</t>
         </is>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="n">
-        <v>12119</v>
+        <v>12145</v>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>3146</t>
+          <t>222</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>CEBOLA GRANULADA</t>
+          <t>CHIMICHURRI FIT</t>
         </is>
       </c>
       <c r="F343" t="inlineStr">
@@ -26832,10 +26832,10 @@
         </is>
       </c>
       <c r="N343" t="n">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="O343" t="n">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="P343" t="n">
         <v>0</v>
@@ -26858,22 +26858,22 @@
       </c>
       <c r="V343" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12119.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12145.webp</t>
         </is>
       </c>
     </row>
     <row r="344">
       <c r="A344" t="n">
-        <v>12115</v>
+        <v>12146</v>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>209</t>
+          <t>304</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>LEMON PEPPER C/ GLUTAMATO</t>
+          <t>CHIMICHURRI C/ PIMENTA FIT</t>
         </is>
       </c>
       <c r="F344" t="inlineStr">
@@ -26909,10 +26909,10 @@
         </is>
       </c>
       <c r="N344" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="O344" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="P344" t="n">
         <v>0</v>
@@ -26935,22 +26935,22 @@
       </c>
       <c r="V344" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12115.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12146.webp</t>
         </is>
       </c>
     </row>
     <row r="345">
       <c r="A345" t="n">
-        <v>12145</v>
+        <v>12147</v>
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>222</t>
+          <t>716</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>CHIMICHURRI FIT</t>
+          <t>LEMON PEPPER FIT</t>
         </is>
       </c>
       <c r="F345" t="inlineStr">
@@ -26986,10 +26986,10 @@
         </is>
       </c>
       <c r="N345" t="n">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="O345" t="n">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="P345" t="n">
         <v>0</v>
@@ -27012,22 +27012,22 @@
       </c>
       <c r="V345" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12145.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12147.jpg</t>
         </is>
       </c>
     </row>
     <row r="346">
       <c r="A346" t="n">
-        <v>12146</v>
+        <v>12148</v>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>304</t>
+          <t>376</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>CHIMICHURRI C/ PIMENTA FIT</t>
+          <t>TEMPERO ANA MARIA FIT</t>
         </is>
       </c>
       <c r="F346" t="inlineStr">
@@ -27063,10 +27063,10 @@
         </is>
       </c>
       <c r="N346" t="n">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="O346" t="n">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="P346" t="n">
         <v>0</v>
@@ -27089,37 +27089,37 @@
       </c>
       <c r="V346" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12146.webp</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12148.jpg</t>
         </is>
       </c>
     </row>
     <row r="347">
       <c r="A347" t="n">
-        <v>12147</v>
+        <v>12160</v>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>716</t>
+          <t>3145</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>LEMON PEPPER FIT</t>
+          <t>MOSTARDA GRAO MARROM 100G</t>
         </is>
       </c>
       <c r="F347" t="inlineStr">
         <is>
-          <t>KG</t>
+          <t>UNID</t>
         </is>
       </c>
       <c r="G347" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="H347" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="I347" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="J347" t="n">
         <v>100</v>
@@ -27140,10 +27140,10 @@
         </is>
       </c>
       <c r="N347" t="n">
-        <v>70</v>
+        <v>5</v>
       </c>
       <c r="O347" t="n">
-        <v>70</v>
+        <v>5</v>
       </c>
       <c r="P347" t="n">
         <v>0</v>
@@ -27157,31 +27157,31 @@
         </is>
       </c>
       <c r="T347" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="U347" t="inlineStr">
         <is>
-          <t>100g</t>
+          <t>UND</t>
         </is>
       </c>
       <c r="V347" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12147.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12160.jpg</t>
         </is>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="n">
-        <v>12148</v>
+        <v>12161</v>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>376</t>
+          <t>1324</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>TEMPERO ANA MARIA FIT</t>
+          <t>NOZ MOSCADA PO CONDIMENTADA</t>
         </is>
       </c>
       <c r="F348" t="inlineStr">
@@ -27217,10 +27217,10 @@
         </is>
       </c>
       <c r="N348" t="n">
-        <v>38</v>
+        <v>160</v>
       </c>
       <c r="O348" t="n">
-        <v>38</v>
+        <v>160</v>
       </c>
       <c r="P348" t="n">
         <v>0</v>
@@ -27243,37 +27243,37 @@
       </c>
       <c r="V348" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12148.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12161.webp</t>
         </is>
       </c>
     </row>
     <row r="349">
       <c r="A349" t="n">
-        <v>12160</v>
+        <v>12164</v>
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>3145</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>MOSTARDA GRAO MARROM 100G</t>
+          <t>PIMENTA JAMAICA (SIRIA PO)</t>
         </is>
       </c>
       <c r="F349" t="inlineStr">
         <is>
-          <t>UNID</t>
+          <t>KG</t>
         </is>
       </c>
       <c r="G349" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="H349" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="I349" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="J349" t="n">
         <v>100</v>
@@ -27294,10 +27294,10 @@
         </is>
       </c>
       <c r="N349" t="n">
-        <v>5</v>
+        <v>85</v>
       </c>
       <c r="O349" t="n">
-        <v>5</v>
+        <v>85</v>
       </c>
       <c r="P349" t="n">
         <v>0</v>
@@ -27311,168 +27311,14 @@
         </is>
       </c>
       <c r="T349" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="U349" t="inlineStr">
         <is>
-          <t>UND</t>
+          <t>100g</t>
         </is>
       </c>
       <c r="V349" t="inlineStr">
-        <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12160.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="350">
-      <c r="A350" t="n">
-        <v>12161</v>
-      </c>
-      <c r="B350" t="inlineStr">
-        <is>
-          <t>1324</t>
-        </is>
-      </c>
-      <c r="C350" t="inlineStr">
-        <is>
-          <t>NOZ MOSCADA PO CONDIMENTADA</t>
-        </is>
-      </c>
-      <c r="F350" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="G350" t="n">
-        <v>10</v>
-      </c>
-      <c r="H350" t="n">
-        <v>10</v>
-      </c>
-      <c r="I350" t="n">
-        <v>5</v>
-      </c>
-      <c r="J350" t="n">
-        <v>100</v>
-      </c>
-      <c r="K350" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L350" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M350" t="inlineStr">
-        <is>
-          <t>TEMPEROS A GRANEL</t>
-        </is>
-      </c>
-      <c r="N350" t="n">
-        <v>160</v>
-      </c>
-      <c r="O350" t="n">
-        <v>160</v>
-      </c>
-      <c r="P350" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q350" t="n">
-        <v>0</v>
-      </c>
-      <c r="S350" t="inlineStr">
-        <is>
-          <t>U</t>
-        </is>
-      </c>
-      <c r="T350" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="U350" t="inlineStr">
-        <is>
-          <t>100g</t>
-        </is>
-      </c>
-      <c r="V350" t="inlineStr">
-        <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12161.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="351">
-      <c r="A351" t="n">
-        <v>12164</v>
-      </c>
-      <c r="B351" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="C351" t="inlineStr">
-        <is>
-          <t>PIMENTA JAMAICA (SIRIA PO)</t>
-        </is>
-      </c>
-      <c r="F351" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="G351" t="n">
-        <v>10</v>
-      </c>
-      <c r="H351" t="n">
-        <v>10</v>
-      </c>
-      <c r="I351" t="n">
-        <v>5</v>
-      </c>
-      <c r="J351" t="n">
-        <v>100</v>
-      </c>
-      <c r="K351" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L351" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M351" t="inlineStr">
-        <is>
-          <t>TEMPEROS A GRANEL</t>
-        </is>
-      </c>
-      <c r="N351" t="n">
-        <v>85</v>
-      </c>
-      <c r="O351" t="n">
-        <v>85</v>
-      </c>
-      <c r="P351" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q351" t="n">
-        <v>0</v>
-      </c>
-      <c r="S351" t="inlineStr">
-        <is>
-          <t>U</t>
-        </is>
-      </c>
-      <c r="T351" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="U351" t="inlineStr">
-        <is>
-          <t>100g</t>
-        </is>
-      </c>
-      <c r="V351" t="inlineStr">
         <is>
           <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/12164.jpg</t>
         </is>

</xml_diff>

<commit_message>
4 trocas verificadas: mandioca/lemon/tamara/aipo
</commit_message>
<xml_diff>
--- a/PLANILHA-FOTOS-NOVAS-355.xlsx
+++ b/PLANILHA-FOTOS-NOVAS-355.xlsx
@@ -11535,7 +11535,7 @@
       </c>
       <c r="V144" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11769.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/farinaceos/11769.jpg</t>
         </is>
       </c>
     </row>
@@ -14230,7 +14230,7 @@
       </c>
       <c r="V179" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11509.jpg</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/frutas-secas/11509.png</t>
         </is>
       </c>
     </row>
@@ -21468,7 +21468,7 @@
       </c>
       <c r="V273" t="inlineStr">
         <is>
-          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11497.png</t>
+          <t>https://rodrigo2612jr.github.io/pascoto-fotos-novas/temperos/11497.jpg</t>
         </is>
       </c>
     </row>

</xml_diff>